<commit_message>
chore(models,ledgers): update calibrated model rating artifacts and daily sport ledgers
</commit_message>
<xml_diff>
--- a/data/sports/cs2/gated.xlsx
+++ b/data/sports/cs2/gated.xlsx
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:DQ144" headerRowCount="1">
-  <autoFilter ref="A1:DQ144"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:DQ150" headerRowCount="1">
+  <autoFilter ref="A1:DQ150"/>
   <tableColumns count="121">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -780,19 +780,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$144)</f>
+        <f>COUNTA('Picks'!$A$2:$A$150)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$144,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$150,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$144,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$150,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$144,"settled",'Picks'!$V$2:$V$144,"win")+COUNTIFS('Picks'!$U$2:$U$144,"settled",'Picks'!$V$2:$V$144,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$150,"settled",'Picks'!$V$2:$V$150,"win")+COUNTIFS('Picks'!$U$2:$U$150,"settled",'Picks'!$V$2:$V$150,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -820,19 +820,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$144,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$150,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$144,"&gt;0",'Picks'!$V$2:$V$144,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$144,"&gt;0",'Picks'!$V$2:$V$144,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$150,"&gt;0",'Picks'!$V$2:$V$150,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$150,"&gt;0",'Picks'!$V$2:$V$150,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$144,"&gt;0",'Picks'!$V$2:$V$144,"win")/(COUNTIFS('Picks'!$BX$2:$BX$144,"&gt;0",'Picks'!$V$2:$V$144,"win")+COUNTIFS('Picks'!$BX$2:$BX$144,"&gt;0",'Picks'!$V$2:$V$144,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$150,"&gt;0",'Picks'!$V$2:$V$150,"win")/(COUNTIFS('Picks'!$BX$2:$BX$150,"&gt;0",'Picks'!$V$2:$V$150,"win")+COUNTIFS('Picks'!$BX$2:$BX$150,"&gt;0",'Picks'!$V$2:$V$150,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$144)/SUM('Picks'!$BX$2:$BX$144),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$150)/SUM('Picks'!$BX$2:$BX$150),0)</f>
         <v/>
       </c>
     </row>
@@ -860,19 +860,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="8">
-        <f>SUM('Picks'!$BY$2:$BY$144)</f>
+        <f>SUM('Picks'!$BY$2:$BY$150)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$144,"&lt;&gt;",'Picks'!$AB$2:$AB$144),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$150,"&lt;&gt;",'Picks'!$AB$2:$AB$150),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$144,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$144,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$150,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$150,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>SUMIFS('Picks'!$AC$2:$AC$144,'Picks'!$AM$2:$AM$144,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$150,'Picks'!$AM$2:$AM$150,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -927,15 +927,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$144,$A14,'Picks'!$U$2:$U$144,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$150,$A14,'Picks'!$U$2:$U$150,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$144,$A14,'Picks'!$U$2:$U$144,"settled",'Picks'!$V$2:$V$144,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$150,$A14,'Picks'!$U$2:$U$150,"settled",'Picks'!$V$2:$V$150,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$144,$A14,'Picks'!$U$2:$U$144,"settled",'Picks'!$V$2:$V$144,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$150,$A14,'Picks'!$U$2:$U$150,"settled",'Picks'!$V$2:$V$150,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -943,11 +943,11 @@
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$144,'Picks'!$H$2:$H$144,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$150,'Picks'!$H$2:$H$150,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$144,'Picks'!$H$2:$H$144,$A14,'Picks'!$U$2:$U$144,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$150,'Picks'!$H$2:$H$150,$A14,'Picks'!$U$2:$U$150,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -958,15 +958,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$144,$A15,'Picks'!$U$2:$U$144,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$150,$A15,'Picks'!$U$2:$U$150,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$144,$A15,'Picks'!$U$2:$U$144,"settled",'Picks'!$V$2:$V$144,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$150,$A15,'Picks'!$U$2:$U$150,"settled",'Picks'!$V$2:$V$150,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$144,$A15,'Picks'!$U$2:$U$144,"settled",'Picks'!$V$2:$V$144,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$150,$A15,'Picks'!$U$2:$U$150,"settled",'Picks'!$V$2:$V$150,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="19">
@@ -974,11 +974,11 @@
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>SUMIFS('Picks'!$BY$2:$BY$144,'Picks'!$H$2:$H$144,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$150,'Picks'!$H$2:$H$150,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$144,'Picks'!$H$2:$H$144,$A15,'Picks'!$U$2:$U$144,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$150,'Picks'!$H$2:$H$150,$A15,'Picks'!$U$2:$U$150,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -989,15 +989,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$144,$A16,'Picks'!$U$2:$U$144,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$150,$A16,'Picks'!$U$2:$U$150,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$144,$A16,'Picks'!$U$2:$U$144,"settled",'Picks'!$V$2:$V$144,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$150,$A16,'Picks'!$U$2:$U$150,"settled",'Picks'!$V$2:$V$150,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$144,$A16,'Picks'!$U$2:$U$144,"settled",'Picks'!$V$2:$V$144,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$150,$A16,'Picks'!$U$2:$U$150,"settled",'Picks'!$V$2:$V$150,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -1005,11 +1005,11 @@
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$144,'Picks'!$H$2:$H$144,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$150,'Picks'!$H$2:$H$150,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$144,'Picks'!$H$2:$H$144,$A16,'Picks'!$U$2:$U$144,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$150,'Picks'!$H$2:$H$150,$A16,'Picks'!$U$2:$U$150,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:DQ144"/>
+  <dimension ref="A1:DQ150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -43623,12 +43623,12 @@
     <row r="133" ht="36" customHeight="1">
       <c r="A133" s="24" t="inlineStr">
         <is>
-          <t>9a4da2e1c7614f01</t>
+          <t>6362a654de014a31</t>
         </is>
       </c>
       <c r="B133" s="24" t="inlineStr">
         <is>
-          <t>2026-10-13T22:38:44.831854Z</t>
+          <t>2026-10-14T06:03:43.455911Z</t>
         </is>
       </c>
       <c r="C133" s="24" t="inlineStr">
@@ -43638,7 +43638,7 @@
       </c>
       <c r="D133" s="24" t="inlineStr">
         <is>
-          <t>157358</t>
+          <t>156607</t>
         </is>
       </c>
       <c r="E133" s="24" t="inlineStr">
@@ -43648,12 +43648,12 @@
       </c>
       <c r="F133" s="24" t="inlineStr">
         <is>
-          <t>Lavked</t>
+          <t>Sökerorg</t>
         </is>
       </c>
       <c r="G133" s="24" t="inlineStr">
         <is>
-          <t>Gothic</t>
+          <t>CTRL Esports</t>
         </is>
       </c>
       <c r="H133" s="24" t="inlineStr">
@@ -43663,7 +43663,7 @@
       </c>
       <c r="I133" s="24" t="inlineStr">
         <is>
-          <t>away</t>
+          <t>home</t>
         </is>
       </c>
       <c r="J133" s="25" t="n"/>
@@ -43673,23 +43673,23 @@
         </is>
       </c>
       <c r="L133" s="26" t="n">
-        <v>-117</v>
+        <v>108</v>
       </c>
       <c r="M133" s="27" t="n">
-        <v>1.854701</v>
+        <v>2.08</v>
       </c>
       <c r="N133" s="28" t="n">
-        <v>0.539171</v>
+        <v>0.480769</v>
       </c>
       <c r="O133" s="28" t="n">
-        <v>0.525718</v>
+        <v>0.531111</v>
       </c>
       <c r="P133" s="28" t="n"/>
       <c r="Q133" s="28" t="n">
-        <v>-0.013453</v>
+        <v>0.050342</v>
       </c>
       <c r="R133" s="26" t="n">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="S133" s="29" t="n">
         <v>1</v>
@@ -43715,7 +43715,7 @@
       <c r="AD133" s="24" t="n"/>
       <c r="AE133" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.5400 (market_slug=aec-cs2-goth-lav-2026-10-14).</t>
+          <t>Neutral Elo baseline; executable ask 0.4800 (market_slug=aec-cs2-cet-skr-2026-10-14).</t>
         </is>
       </c>
       <c r="AF133" s="31" t="inlineStr">
@@ -43751,37 +43751,37 @@
       </c>
       <c r="AO133" s="24" t="inlineStr">
         <is>
-          <t>PAPER_CALL_LOW_EDGE</t>
+          <t>PAPER_CALL_MODEL_UNVALIDATED</t>
         </is>
       </c>
       <c r="AP133" s="24" t="inlineStr">
         <is>
-          <t>Lavked</t>
+          <t>Sökerorg</t>
         </is>
       </c>
       <c r="AQ133" s="24" t="inlineStr">
         <is>
-          <t>Lavked</t>
+          <t>Sökerorg</t>
         </is>
       </c>
       <c r="AR133" s="24" t="inlineStr">
         <is>
-          <t>Lavked</t>
+          <t>Sökerorg</t>
         </is>
       </c>
       <c r="AS133" s="24" t="inlineStr">
         <is>
-          <t>Gothic</t>
+          <t>CTRL Esports</t>
         </is>
       </c>
       <c r="AT133" s="24" t="inlineStr">
         <is>
-          <t>Gothic</t>
+          <t>CTRL Esports</t>
         </is>
       </c>
       <c r="AU133" s="24" t="inlineStr">
         <is>
-          <t>Gothic</t>
+          <t>CTRL Esports</t>
         </is>
       </c>
       <c r="AV133" s="24" t="n"/>
@@ -43799,7 +43799,7 @@
       </c>
       <c r="BA133" s="24" t="inlineStr">
         <is>
-          <t>21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5</t>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
         </is>
       </c>
       <c r="BB133" s="24" t="inlineStr">
@@ -43814,7 +43814,7 @@
       </c>
       <c r="BD133" s="24" t="inlineStr">
         <is>
-          <t>21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5</t>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
         </is>
       </c>
       <c r="BE133" s="24" t="inlineStr">
@@ -43834,7 +43834,7 @@
       </c>
       <c r="BH133" s="24" t="inlineStr">
         <is>
-          <t>2026-10-13T22:30:28.144639Z</t>
+          <t>2026-10-14T05:52:34.675602Z</t>
         </is>
       </c>
       <c r="BI133" s="24" t="inlineStr">
@@ -43844,13 +43844,13 @@
       </c>
       <c r="BJ133" s="25" t="n"/>
       <c r="BK133" s="26" t="n">
-        <v>-117</v>
+        <v>108</v>
       </c>
       <c r="BL133" s="27" t="n">
-        <v>1.854701</v>
+        <v>2.08</v>
       </c>
       <c r="BM133" s="28" t="n">
-        <v>0.539171</v>
+        <v>0.480769</v>
       </c>
       <c r="BN133" s="28" t="n"/>
       <c r="BO133" s="28" t="n"/>
@@ -43885,7 +43885,7 @@
       <c r="CR133" s="24" t="n"/>
       <c r="CS133" s="24" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="CT133" s="24" t="n"/>
@@ -43913,19 +43913,19 @@
       <c r="DP133" s="24" t="n"/>
       <c r="DQ133" s="24" t="inlineStr">
         <is>
-          <t>{"artifact_hash": "21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5", "away_team": "Lavked", "event_id": "157358", "event_start_utc": "2026-10-14T08:00:00Z", "features": {"away_elo": 1562.723044, "away_history_count": 122, "home_elo": 1519.966768, "home_history_count": 7}, "historical_source_observation_times_verified": false, "home_team": "Gothic", "inference_inputs": {"book_state": {"games_played": {"bo3:1:23078": 122, "bo3:1:25275": 7}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 40.0, "last_match_utc": {"bo3:1:23078": "2026-10-11T17:10:00Z", "bo3:1:25275": "2026-10-11T11:00:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.06816528215678655, "platt_slope": 0.8746273142827576, "ratings": {"bo3:1:23078": 1562.723044, "bo3:1:25275": 1519.966768}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "8d25951d04320147b4f82f35408c7948ac3d6a80af203ada3bac1aa630e7b330", "features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872"}, "reference_date": "2026-10-13T22:29:07.911078+00:00", "team_ids": ["bo3:1:25275", "bo3:1:23078"]}, "market_type": "moneyline", "model_version": "cs2-tiered-elo-v6", "observed_at_utc": "2026-10-13T22:29:07.911078+00:00", "probabilities": {"away": 0.525718, "home": 0.474282}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "38470c58dfdf2ab5b6defadd5fd729bee2e1b52f764d45bf2f093eb2198df0fb", "sport": "CS2"}</t>
+          <t>{"artifact_hash": "642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7", "away_team": "S\u00f6kerorg", "event_id": "156607", "event_start_utc": "2026-10-14T08:00:00Z", "features": {"away_elo": 1452.531883, "away_history_count": 4, "home_elo": 1500.0, "home_history_count": 0}, "historical_source_observation_times_verified": false, "home_team": "CTRL Esports", "inference_inputs": {"book_state": {"games_played": {"bo3:1:25400": 4}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 40.0, "last_match_utc": {"bo3:1:25400": "2026-10-08T13:00:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.06821870672347567, "platt_slope": 0.8748911450799665, "ratings": {"bo3:1:25400": 1452.531883}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "3abbfc5d7124cc94603dada2e4c996da231a679d437c5a066d994a2a7d428f61", "features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872"}, "reference_date": "2026-10-14T05:52:14.154858+00:00", "team_ids": ["unknown:ctrlesports", "bo3:1:25400"]}, "market_type": "moneyline", "model_version": "cs2-tiered-elo-v6", "observed_at_utc": "2026-10-14T05:52:14.154858+00:00", "probabilities": {"away": 0.468889, "home": 0.531111}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "8e9aafb743ee4bf33e66088136495d0001915ef2177d4e7411823bae9de7cd2f", "sport": "CS2"}</t>
         </is>
       </c>
     </row>
     <row r="134" ht="36" customHeight="1">
       <c r="A134" s="24" t="inlineStr">
         <is>
-          <t>dedcf70ef92b4c53</t>
+          <t>c42dc0256c3d4450</t>
         </is>
       </c>
       <c r="B134" s="24" t="inlineStr">
         <is>
-          <t>2026-10-13T22:38:44.831854Z</t>
+          <t>2026-10-14T06:03:43.455911Z</t>
         </is>
       </c>
       <c r="C134" s="24" t="inlineStr">
@@ -43935,7 +43935,7 @@
       </c>
       <c r="D134" s="24" t="inlineStr">
         <is>
-          <t>157861</t>
+          <t>156906</t>
         </is>
       </c>
       <c r="E134" s="24" t="inlineStr">
@@ -43945,12 +43945,12 @@
       </c>
       <c r="F134" s="24" t="inlineStr">
         <is>
-          <t>6666</t>
+          <t>B8 Academy</t>
         </is>
       </c>
       <c r="G134" s="24" t="inlineStr">
         <is>
-          <t>GenOne</t>
+          <t>ENJOY</t>
         </is>
       </c>
       <c r="H134" s="24" t="inlineStr">
@@ -43970,20 +43970,20 @@
         </is>
       </c>
       <c r="L134" s="26" t="n">
-        <v>-163</v>
+        <v>-170</v>
       </c>
       <c r="M134" s="27" t="n">
-        <v>1.613497</v>
+        <v>1.588235</v>
       </c>
       <c r="N134" s="28" t="n">
-        <v>0.619772</v>
+        <v>0.62963</v>
       </c>
       <c r="O134" s="28" t="n">
-        <v>0.502013</v>
+        <v>0.550806</v>
       </c>
       <c r="P134" s="28" t="n"/>
       <c r="Q134" s="28" t="n">
-        <v>-0.117759</v>
+        <v>-0.07882400000000001</v>
       </c>
       <c r="R134" s="26" t="n">
         <v>0</v>
@@ -44012,7 +44012,7 @@
       <c r="AD134" s="24" t="n"/>
       <c r="AE134" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.6200 (market_slug=aec-cs2-g1-6666-2026-10-14).</t>
+          <t>Neutral Elo baseline; executable ask 0.6300 (market_slug=aec-cs2-enjoy-b8a-2026-10-14).</t>
         </is>
       </c>
       <c r="AF134" s="31" t="inlineStr">
@@ -44053,32 +44053,32 @@
       </c>
       <c r="AP134" s="24" t="inlineStr">
         <is>
-          <t>6666</t>
+          <t>B8 Academy</t>
         </is>
       </c>
       <c r="AQ134" s="24" t="inlineStr">
         <is>
-          <t>6666</t>
+          <t>B8 Academy</t>
         </is>
       </c>
       <c r="AR134" s="24" t="inlineStr">
         <is>
-          <t>6666</t>
+          <t>B8 Academy</t>
         </is>
       </c>
       <c r="AS134" s="24" t="inlineStr">
         <is>
-          <t>GenOne</t>
+          <t>ENJOY</t>
         </is>
       </c>
       <c r="AT134" s="24" t="inlineStr">
         <is>
-          <t>GenOne</t>
+          <t>ENJOY</t>
         </is>
       </c>
       <c r="AU134" s="24" t="inlineStr">
         <is>
-          <t>GenOne</t>
+          <t>ENJOY</t>
         </is>
       </c>
       <c r="AV134" s="24" t="n"/>
@@ -44096,7 +44096,7 @@
       </c>
       <c r="BA134" s="24" t="inlineStr">
         <is>
-          <t>21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5</t>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
         </is>
       </c>
       <c r="BB134" s="24" t="inlineStr">
@@ -44111,7 +44111,7 @@
       </c>
       <c r="BD134" s="24" t="inlineStr">
         <is>
-          <t>21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5</t>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
         </is>
       </c>
       <c r="BE134" s="24" t="inlineStr">
@@ -44131,7 +44131,7 @@
       </c>
       <c r="BH134" s="24" t="inlineStr">
         <is>
-          <t>2026-10-13T22:30:48.854407Z</t>
+          <t>2026-10-14T05:53:04.500324Z</t>
         </is>
       </c>
       <c r="BI134" s="24" t="inlineStr">
@@ -44141,13 +44141,13 @@
       </c>
       <c r="BJ134" s="25" t="n"/>
       <c r="BK134" s="26" t="n">
-        <v>-163</v>
+        <v>-170</v>
       </c>
       <c r="BL134" s="27" t="n">
-        <v>1.613497</v>
+        <v>1.588235</v>
       </c>
       <c r="BM134" s="28" t="n">
-        <v>0.619772</v>
+        <v>0.62963</v>
       </c>
       <c r="BN134" s="28" t="n"/>
       <c r="BO134" s="28" t="n"/>
@@ -44210,29 +44210,29 @@
       <c r="DP134" s="24" t="n"/>
       <c r="DQ134" s="24" t="inlineStr">
         <is>
-          <t>{"artifact_hash": "21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5", "away_team": "6666", "event_id": "157861", "event_start_utc": "2026-10-14T08:00:00Z", "features": {"away_elo": 1681.928565, "away_history_count": 38, "home_elo": 1671.902053, "home_history_count": 472}, "historical_source_observation_times_verified": false, "home_team": "GenOne", "inference_inputs": {"book_state": {"games_played": {"bo3:1:1406": 472, "bo3:1:24507": 38}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 40.0, "last_match_utc": {"bo3:1:1406": "2026-10-12T15:50:00Z", "bo3:1:24507": "2026-10-13T17:00:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.06816528215678655, "platt_slope": 0.8746273142827576, "ratings": {"bo3:1:1406": 1671.902053, "bo3:1:24507": 1681.928565}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "8d25951d04320147b4f82f35408c7948ac3d6a80af203ada3bac1aa630e7b330", "features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872"}, "reference_date": "2026-10-13T22:29:07.911078+00:00", "team_ids": ["bo3:1:1406", "bo3:1:24507"]}, "market_type": "moneyline", "model_version": "cs2-tiered-elo-v6", "observed_at_utc": "2026-10-13T22:29:07.911078+00:00", "probabilities": {"away": 0.497987, "home": 0.502013}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "dd88004fc423e84f3129a72adfb257fe3e5acb95e801068956a3affa355b4ebd", "sport": "CS2"}</t>
+          <t>{"artifact_hash": "642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7", "away_team": "B8 Academy", "event_id": "156906", "event_start_utc": "2026-10-14T08:00:00Z", "features": {"away_elo": 1482.405877, "away_history_count": 84, "home_elo": 1517.818023, "home_history_count": 85}, "historical_source_observation_times_verified": false, "home_team": "ENJOY", "inference_inputs": {"book_state": {"games_played": {"bo3:1:10966": 85, "bo3:1:21936": 84}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 40.0, "last_match_utc": {"bo3:1:10966": "2026-10-12T08:10:00Z", "bo3:1:21936": "2026-10-08T16:10:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.06821870672347567, "platt_slope": 0.8748911450799665, "ratings": {"bo3:1:10966": 1517.818023, "bo3:1:21936": 1482.405877}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "3abbfc5d7124cc94603dada2e4c996da231a679d437c5a066d994a2a7d428f61", "features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872"}, "reference_date": "2026-10-14T05:52:14.154858+00:00", "team_ids": ["bo3:1:10966", "bo3:1:21936"]}, "market_type": "moneyline", "model_version": "cs2-tiered-elo-v6", "observed_at_utc": "2026-10-14T05:52:14.154858+00:00", "probabilities": {"away": 0.449194, "home": 0.550806}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "eea90a6e62a45839d43ed6441191eb36ba08555e1c31533996ab8bcbe9ea8bb8", "sport": "CS2"}</t>
         </is>
       </c>
     </row>
     <row r="135" ht="36" customHeight="1">
       <c r="A135" s="24" t="inlineStr">
         <is>
-          <t>84c1e4e967e5471e</t>
+          <t>3f887828ca054cfe</t>
         </is>
       </c>
       <c r="B135" s="24" t="inlineStr">
         <is>
-          <t>2026-10-13T22:38:44.831854Z</t>
+          <t>2026-10-14T06:03:43.455911Z</t>
         </is>
       </c>
       <c r="C135" s="24" t="inlineStr">
         <is>
-          <t>2026-10-14T08:30:00Z</t>
+          <t>2026-10-14T08:00:00Z</t>
         </is>
       </c>
       <c r="D135" s="24" t="inlineStr">
         <is>
-          <t>154535</t>
+          <t>157358</t>
         </is>
       </c>
       <c r="E135" s="24" t="inlineStr">
@@ -44242,12 +44242,12 @@
       </c>
       <c r="F135" s="24" t="inlineStr">
         <is>
-          <t>Aurora Gaming</t>
+          <t>Lavked</t>
         </is>
       </c>
       <c r="G135" s="24" t="inlineStr">
         <is>
-          <t>9z</t>
+          <t>Gothic</t>
         </is>
       </c>
       <c r="H135" s="24" t="inlineStr">
@@ -44269,20 +44269,20 @@
         </is>
       </c>
       <c r="L135" s="26" t="n">
-        <v>-163</v>
+        <v>-127</v>
       </c>
       <c r="M135" s="27" t="n">
-        <v>1.613497</v>
+        <v>1.787402</v>
       </c>
       <c r="N135" s="28" t="n">
-        <v>0.619772</v>
+        <v>0.5594710000000001</v>
       </c>
       <c r="O135" s="28" t="n">
-        <v>0.548671</v>
+        <v>0.500583</v>
       </c>
       <c r="P135" s="28" t="n"/>
       <c r="Q135" s="28" t="n">
-        <v>-0.071101</v>
+        <v>-0.058888</v>
       </c>
       <c r="R135" s="26" t="n">
         <v>0</v>
@@ -44311,7 +44311,7 @@
       <c r="AD135" s="24" t="n"/>
       <c r="AE135" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.6200 (market_slug=tsc-cs2-9z-aur-2026-10-14-tot-2pt5).</t>
+          <t>Neutral Elo baseline; executable ask 0.5600 (market_slug=tsc-cs2-goth-lav-2026-10-14-tot-2pt5).</t>
         </is>
       </c>
       <c r="AF135" s="31" t="inlineStr">
@@ -44352,32 +44352,32 @@
       </c>
       <c r="AP135" s="24" t="inlineStr">
         <is>
-          <t>Aurora Gaming</t>
+          <t>Lavked</t>
         </is>
       </c>
       <c r="AQ135" s="24" t="inlineStr">
         <is>
-          <t>Aurora Gaming</t>
+          <t>Lavked</t>
         </is>
       </c>
       <c r="AR135" s="24" t="inlineStr">
         <is>
-          <t>Aurora Gaming</t>
+          <t>Lavked</t>
         </is>
       </c>
       <c r="AS135" s="24" t="inlineStr">
         <is>
-          <t>9z</t>
+          <t>Gothic</t>
         </is>
       </c>
       <c r="AT135" s="24" t="inlineStr">
         <is>
-          <t>9z</t>
+          <t>Gothic</t>
         </is>
       </c>
       <c r="AU135" s="24" t="inlineStr">
         <is>
-          <t>9z</t>
+          <t>Gothic</t>
         </is>
       </c>
       <c r="AV135" s="24" t="n"/>
@@ -44395,7 +44395,7 @@
       </c>
       <c r="BA135" s="24" t="inlineStr">
         <is>
-          <t>21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5</t>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
         </is>
       </c>
       <c r="BB135" s="24" t="inlineStr">
@@ -44410,7 +44410,7 @@
       </c>
       <c r="BD135" s="24" t="inlineStr">
         <is>
-          <t>21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5</t>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
         </is>
       </c>
       <c r="BE135" s="24" t="inlineStr">
@@ -44430,7 +44430,7 @@
       </c>
       <c r="BH135" s="24" t="inlineStr">
         <is>
-          <t>2026-10-13T22:31:19.935072Z</t>
+          <t>2026-10-14T05:53:46.757629Z</t>
         </is>
       </c>
       <c r="BI135" s="24" t="inlineStr">
@@ -44442,13 +44442,13 @@
         <v>2.5</v>
       </c>
       <c r="BK135" s="26" t="n">
-        <v>-163</v>
+        <v>-127</v>
       </c>
       <c r="BL135" s="27" t="n">
-        <v>1.613497</v>
+        <v>1.787402</v>
       </c>
       <c r="BM135" s="28" t="n">
-        <v>0.619772</v>
+        <v>0.5594710000000001</v>
       </c>
       <c r="BN135" s="28" t="n"/>
       <c r="BO135" s="28" t="n"/>
@@ -44514,22 +44514,22 @@
     <row r="136" ht="36" customHeight="1">
       <c r="A136" s="24" t="inlineStr">
         <is>
-          <t>9f2258f06cd843b1</t>
+          <t>0adc75eeb0344b58</t>
         </is>
       </c>
       <c r="B136" s="24" t="inlineStr">
         <is>
-          <t>2026-10-13T22:38:44.831854Z</t>
+          <t>2026-10-14T06:03:43.455911Z</t>
         </is>
       </c>
       <c r="C136" s="24" t="inlineStr">
         <is>
-          <t>2026-10-14T10:00:00Z</t>
+          <t>2026-10-14T10:30:00Z</t>
         </is>
       </c>
       <c r="D136" s="24" t="inlineStr">
         <is>
-          <t>154600</t>
+          <t>156609</t>
         </is>
       </c>
       <c r="E136" s="24" t="inlineStr">
@@ -44539,12 +44539,12 @@
       </c>
       <c r="F136" s="24" t="inlineStr">
         <is>
-          <t>fnatic</t>
+          <t>Bread Eaters Esports</t>
         </is>
       </c>
       <c r="G136" s="24" t="inlineStr">
         <is>
-          <t>HOTU</t>
+          <t>EAC Extra</t>
         </is>
       </c>
       <c r="H136" s="24" t="inlineStr">
@@ -44566,20 +44566,20 @@
         </is>
       </c>
       <c r="L136" s="26" t="n">
-        <v>-127</v>
+        <v>-138</v>
       </c>
       <c r="M136" s="27" t="n">
-        <v>1.787402</v>
+        <v>1.724638</v>
       </c>
       <c r="N136" s="28" t="n">
-        <v>0.5594710000000001</v>
+        <v>0.579832</v>
       </c>
       <c r="O136" s="28" t="n">
-        <v>0.500099</v>
+        <v>0.501205</v>
       </c>
       <c r="P136" s="28" t="n"/>
       <c r="Q136" s="28" t="n">
-        <v>-0.059372</v>
+        <v>-0.078627</v>
       </c>
       <c r="R136" s="26" t="n">
         <v>0</v>
@@ -44608,7 +44608,7 @@
       <c r="AD136" s="24" t="n"/>
       <c r="AE136" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.5600 (market_slug=tsc-cs2-hotu-fnc-2026-10-14-tot-2pt5).</t>
+          <t>Neutral Elo baseline; executable ask 0.5800 (market_slug=tsc-cs2-eace-bee-2026-10-14-tot-2pt5).</t>
         </is>
       </c>
       <c r="AF136" s="31" t="inlineStr">
@@ -44649,32 +44649,32 @@
       </c>
       <c r="AP136" s="24" t="inlineStr">
         <is>
-          <t>fnatic</t>
+          <t>Bread Eaters Esports</t>
         </is>
       </c>
       <c r="AQ136" s="24" t="inlineStr">
         <is>
-          <t>fnatic</t>
+          <t>Bread Eaters Esports</t>
         </is>
       </c>
       <c r="AR136" s="24" t="inlineStr">
         <is>
-          <t>fnatic</t>
+          <t>Bread Eaters Esports</t>
         </is>
       </c>
       <c r="AS136" s="24" t="inlineStr">
         <is>
-          <t>HOTU</t>
+          <t>EAC Extra</t>
         </is>
       </c>
       <c r="AT136" s="24" t="inlineStr">
         <is>
-          <t>HOTU</t>
+          <t>EAC Extra</t>
         </is>
       </c>
       <c r="AU136" s="24" t="inlineStr">
         <is>
-          <t>HOTU</t>
+          <t>EAC Extra</t>
         </is>
       </c>
       <c r="AV136" s="24" t="n"/>
@@ -44692,7 +44692,7 @@
       </c>
       <c r="BA136" s="24" t="inlineStr">
         <is>
-          <t>21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5</t>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
         </is>
       </c>
       <c r="BB136" s="24" t="inlineStr">
@@ -44707,7 +44707,7 @@
       </c>
       <c r="BD136" s="24" t="inlineStr">
         <is>
-          <t>21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5</t>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
         </is>
       </c>
       <c r="BE136" s="24" t="inlineStr">
@@ -44727,7 +44727,7 @@
       </c>
       <c r="BH136" s="24" t="inlineStr">
         <is>
-          <t>2026-10-13T22:32:22.495588Z</t>
+          <t>2026-10-14T05:56:43.658008Z</t>
         </is>
       </c>
       <c r="BI136" s="24" t="inlineStr">
@@ -44739,13 +44739,13 @@
         <v>2.5</v>
       </c>
       <c r="BK136" s="26" t="n">
-        <v>-127</v>
+        <v>-138</v>
       </c>
       <c r="BL136" s="27" t="n">
-        <v>1.787402</v>
+        <v>1.724638</v>
       </c>
       <c r="BM136" s="28" t="n">
-        <v>0.5594710000000001</v>
+        <v>0.579832</v>
       </c>
       <c r="BN136" s="28" t="n"/>
       <c r="BO136" s="28" t="n"/>
@@ -44811,22 +44811,22 @@
     <row r="137" ht="36" customHeight="1">
       <c r="A137" s="24" t="inlineStr">
         <is>
-          <t>fd29d257ac074910</t>
+          <t>dbf90710cdd3450d</t>
         </is>
       </c>
       <c r="B137" s="24" t="inlineStr">
         <is>
-          <t>2026-10-13T22:38:44.831854Z</t>
+          <t>2026-10-14T06:03:43.455911Z</t>
         </is>
       </c>
       <c r="C137" s="24" t="inlineStr">
         <is>
-          <t>2026-10-14T10:00:00Z</t>
+          <t>2026-10-14T11:00:00Z</t>
         </is>
       </c>
       <c r="D137" s="24" t="inlineStr">
         <is>
-          <t>154600</t>
+          <t>154657</t>
         </is>
       </c>
       <c r="E137" s="24" t="inlineStr">
@@ -44836,55 +44836,57 @@
       </c>
       <c r="F137" s="24" t="inlineStr">
         <is>
-          <t>fnatic</t>
+          <t>NIP</t>
         </is>
       </c>
       <c r="G137" s="24" t="inlineStr">
         <is>
-          <t>HOTU</t>
+          <t>Team Falcons</t>
         </is>
       </c>
       <c r="H137" s="24" t="inlineStr">
         <is>
-          <t>moneyline</t>
+          <t>total</t>
         </is>
       </c>
       <c r="I137" s="24" t="inlineStr">
         <is>
-          <t>away</t>
-        </is>
-      </c>
-      <c r="J137" s="25" t="n"/>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="J137" s="25" t="n">
+        <v>2.5</v>
+      </c>
       <c r="K137" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
         </is>
       </c>
       <c r="L137" s="26" t="n">
-        <v>-117</v>
+        <v>-150</v>
       </c>
       <c r="M137" s="27" t="n">
-        <v>1.854701</v>
+        <v>1.666667</v>
       </c>
       <c r="N137" s="28" t="n">
-        <v>0.539171</v>
+        <v>0.6</v>
       </c>
       <c r="O137" s="28" t="n">
-        <v>0.510527</v>
+        <v>0.54065</v>
       </c>
       <c r="P137" s="28" t="n"/>
       <c r="Q137" s="28" t="n">
-        <v>-0.028644</v>
+        <v>-0.05935</v>
       </c>
       <c r="R137" s="26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S137" s="29" t="n">
         <v>1</v>
       </c>
       <c r="T137" s="24" t="inlineStr">
         <is>
-          <t>cs2-tiered-elo-v6</t>
+          <t>cs2-total-tiered-elo-v6</t>
         </is>
       </c>
       <c r="U137" s="24" t="inlineStr">
@@ -44903,7 +44905,7 @@
       <c r="AD137" s="24" t="n"/>
       <c r="AE137" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.5400 (market_slug=aec-cs2-hotu-fnc-2026-10-14).</t>
+          <t>Neutral Elo baseline; executable ask 0.6000 (market_slug=tsc-cs2-fal-nip-2026-10-14-tot-2pt5).</t>
         </is>
       </c>
       <c r="AF137" s="31" t="inlineStr">
@@ -44944,32 +44946,32 @@
       </c>
       <c r="AP137" s="24" t="inlineStr">
         <is>
-          <t>fnatic</t>
+          <t>NIP</t>
         </is>
       </c>
       <c r="AQ137" s="24" t="inlineStr">
         <is>
-          <t>fnatic</t>
+          <t>NIP</t>
         </is>
       </c>
       <c r="AR137" s="24" t="inlineStr">
         <is>
-          <t>fnatic</t>
+          <t>NIP</t>
         </is>
       </c>
       <c r="AS137" s="24" t="inlineStr">
         <is>
-          <t>HOTU</t>
+          <t>Team Falcons</t>
         </is>
       </c>
       <c r="AT137" s="24" t="inlineStr">
         <is>
-          <t>HOTU</t>
+          <t>Team Falcons</t>
         </is>
       </c>
       <c r="AU137" s="24" t="inlineStr">
         <is>
-          <t>HOTU</t>
+          <t>Team Falcons</t>
         </is>
       </c>
       <c r="AV137" s="24" t="n"/>
@@ -44987,7 +44989,7 @@
       </c>
       <c r="BA137" s="24" t="inlineStr">
         <is>
-          <t>21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5</t>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
         </is>
       </c>
       <c r="BB137" s="24" t="inlineStr">
@@ -44997,12 +44999,12 @@
       </c>
       <c r="BC137" s="24" t="inlineStr">
         <is>
-          <t>cs2-tiered-elo-v6</t>
+          <t>cs2-total-tiered-elo-v6</t>
         </is>
       </c>
       <c r="BD137" s="24" t="inlineStr">
         <is>
-          <t>21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5</t>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
         </is>
       </c>
       <c r="BE137" s="24" t="inlineStr">
@@ -45017,12 +45019,12 @@
       </c>
       <c r="BG137" s="24" t="inlineStr">
         <is>
-          <t>cs2-tiered-elo-v6</t>
+          <t>cs2-total-tiered-elo-v6</t>
         </is>
       </c>
       <c r="BH137" s="24" t="inlineStr">
         <is>
-          <t>2026-10-13T22:32:22.553820Z</t>
+          <t>2026-10-14T05:57:14.991445Z</t>
         </is>
       </c>
       <c r="BI137" s="24" t="inlineStr">
@@ -45030,15 +45032,17 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ137" s="25" t="n"/>
+      <c r="BJ137" s="25" t="n">
+        <v>2.5</v>
+      </c>
       <c r="BK137" s="26" t="n">
-        <v>-117</v>
+        <v>-150</v>
       </c>
       <c r="BL137" s="27" t="n">
-        <v>1.854701</v>
+        <v>1.666667</v>
       </c>
       <c r="BM137" s="28" t="n">
-        <v>0.539171</v>
+        <v>0.6</v>
       </c>
       <c r="BN137" s="28" t="n"/>
       <c r="BO137" s="28" t="n"/>
@@ -45099,31 +45103,27 @@
       <c r="DN137" s="24" t="n"/>
       <c r="DO137" s="24" t="n"/>
       <c r="DP137" s="24" t="n"/>
-      <c r="DQ137" s="24" t="inlineStr">
-        <is>
-          <t>{"artifact_hash": "21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5", "away_team": "fnatic", "event_id": "154600", "event_start_utc": "2026-10-14T10:00:00Z", "features": {"away_elo": 1927.166299, "away_history_count": 322, "home_elo": 1902.991706, "home_history_count": 267}, "historical_source_observation_times_verified": false, "home_team": "HOTU", "inference_inputs": {"book_state": {"games_played": {"bo3:1:2720": 267, "bo3:1:786": 322}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 40.0, "last_match_utc": {"bo3:1:2720": "2026-10-10T10:00:00Z", "bo3:1:786": "2026-10-10T10:00:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.06816528215678655, "platt_slope": 0.8746273142827576, "ratings": {"bo3:1:2720": 1902.991706, "bo3:1:786": 1927.166299}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "8d25951d04320147b4f82f35408c7948ac3d6a80af203ada3bac1aa630e7b330", "features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872"}, "reference_date": "2026-10-13T22:29:07.911078+00:00", "team_ids": ["bo3:1:2720", "bo3:1:786"]}, "market_type": "moneyline", "model_version": "cs2-tiered-elo-v6", "observed_at_utc": "2026-10-13T22:29:07.911078+00:00", "probabilities": {"away": 0.510527, "home": 0.489473}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "55b27ab49774f2cfed2350503a772c977dd0496ccbb56a77d48d970aa3f564a8", "sport": "CS2"}</t>
-        </is>
-      </c>
+      <c r="DQ137" s="24" t="n"/>
     </row>
     <row r="138" ht="36" customHeight="1">
       <c r="A138" s="24" t="inlineStr">
         <is>
-          <t>55da60c243cb4b26</t>
+          <t>6604a360d3db47c0</t>
         </is>
       </c>
       <c r="B138" s="24" t="inlineStr">
         <is>
-          <t>2026-10-13T22:38:44.831854Z</t>
+          <t>2026-10-14T06:03:43.455911Z</t>
         </is>
       </c>
       <c r="C138" s="24" t="inlineStr">
         <is>
-          <t>2026-10-14T10:30:00Z</t>
+          <t>2026-10-14T11:00:00Z</t>
         </is>
       </c>
       <c r="D138" s="24" t="inlineStr">
         <is>
-          <t>156609</t>
+          <t>156908</t>
         </is>
       </c>
       <c r="E138" s="24" t="inlineStr">
@@ -45133,12 +45133,12 @@
       </c>
       <c r="F138" s="24" t="inlineStr">
         <is>
-          <t>Bread Eaters Esports</t>
+          <t>6666</t>
         </is>
       </c>
       <c r="G138" s="24" t="inlineStr">
         <is>
-          <t>EAC Extra</t>
+          <t>los kogutos</t>
         </is>
       </c>
       <c r="H138" s="24" t="inlineStr">
@@ -45148,7 +45148,7 @@
       </c>
       <c r="I138" s="24" t="inlineStr">
         <is>
-          <t>home</t>
+          <t>away</t>
         </is>
       </c>
       <c r="J138" s="25" t="n"/>
@@ -45158,26 +45158,26 @@
         </is>
       </c>
       <c r="L138" s="26" t="n">
-        <v>-170</v>
+        <v>117</v>
       </c>
       <c r="M138" s="27" t="n">
-        <v>1.588235</v>
+        <v>2.17</v>
       </c>
       <c r="N138" s="28" t="n">
-        <v>0.62963</v>
+        <v>0.460829</v>
       </c>
       <c r="O138" s="28" t="n">
-        <v>0.53684</v>
+        <v>0.650526</v>
       </c>
       <c r="P138" s="28" t="n"/>
       <c r="Q138" s="28" t="n">
-        <v>-0.09279</v>
+        <v>0.189697</v>
       </c>
       <c r="R138" s="26" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S138" s="29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T138" s="24" t="inlineStr">
         <is>
@@ -45200,7 +45200,7 @@
       <c r="AD138" s="24" t="n"/>
       <c r="AE138" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.6300 (market_slug=aec-cs2-eace-bee-2026-10-14).</t>
+          <t>Neutral Elo baseline; executable ask 0.4600 (market_slug=aec-cs2-lk-6666-2026-10-14).</t>
         </is>
       </c>
       <c r="AF138" s="31" t="inlineStr">
@@ -45218,7 +45218,7 @@
       <c r="AJ138" s="31" t="n"/>
       <c r="AK138" s="24" t="inlineStr">
         <is>
-          <t>paper_call</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL138" s="26" t="n">
@@ -45226,7 +45226,7 @@
       </c>
       <c r="AM138" s="24" t="inlineStr">
         <is>
-          <t>RESEARCH_OBSERVATION</t>
+          <t>QUALIFIED_SHADOW_CALL</t>
         </is>
       </c>
       <c r="AN138" s="24" t="inlineStr">
@@ -45236,37 +45236,37 @@
       </c>
       <c r="AO138" s="24" t="inlineStr">
         <is>
-          <t>PAPER_CALL_LOW_EDGE</t>
+          <t>QUALIFIED</t>
         </is>
       </c>
       <c r="AP138" s="24" t="inlineStr">
         <is>
-          <t>Bread Eaters Esports</t>
+          <t>6666</t>
         </is>
       </c>
       <c r="AQ138" s="24" t="inlineStr">
         <is>
-          <t>Bread Eaters Esports</t>
+          <t>6666</t>
         </is>
       </c>
       <c r="AR138" s="24" t="inlineStr">
         <is>
-          <t>Bread Eaters Esports</t>
+          <t>6666</t>
         </is>
       </c>
       <c r="AS138" s="24" t="inlineStr">
         <is>
-          <t>EAC Extra</t>
+          <t>los kogutos</t>
         </is>
       </c>
       <c r="AT138" s="24" t="inlineStr">
         <is>
-          <t>EAC Extra</t>
+          <t>los kogutos</t>
         </is>
       </c>
       <c r="AU138" s="24" t="inlineStr">
         <is>
-          <t>EAC Extra</t>
+          <t>los kogutos</t>
         </is>
       </c>
       <c r="AV138" s="24" t="n"/>
@@ -45284,7 +45284,7 @@
       </c>
       <c r="BA138" s="24" t="inlineStr">
         <is>
-          <t>21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5</t>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
         </is>
       </c>
       <c r="BB138" s="24" t="inlineStr">
@@ -45299,7 +45299,7 @@
       </c>
       <c r="BD138" s="24" t="inlineStr">
         <is>
-          <t>21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5</t>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
         </is>
       </c>
       <c r="BE138" s="24" t="inlineStr">
@@ -45319,7 +45319,7 @@
       </c>
       <c r="BH138" s="24" t="inlineStr">
         <is>
-          <t>2026-10-13T22:33:33.948006Z</t>
+          <t>2026-10-14T05:57:56.430521Z</t>
         </is>
       </c>
       <c r="BI138" s="24" t="inlineStr">
@@ -45329,13 +45329,13 @@
       </c>
       <c r="BJ138" s="25" t="n"/>
       <c r="BK138" s="26" t="n">
-        <v>-170</v>
+        <v>117</v>
       </c>
       <c r="BL138" s="27" t="n">
-        <v>1.588235</v>
+        <v>2.17</v>
       </c>
       <c r="BM138" s="28" t="n">
-        <v>0.62963</v>
+        <v>0.460829</v>
       </c>
       <c r="BN138" s="28" t="n"/>
       <c r="BO138" s="28" t="n"/>
@@ -45370,7 +45370,7 @@
       <c r="CR138" s="24" t="n"/>
       <c r="CS138" s="24" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="CT138" s="24" t="n"/>
@@ -45398,19 +45398,19 @@
       <c r="DP138" s="24" t="n"/>
       <c r="DQ138" s="24" t="inlineStr">
         <is>
-          <t>{"artifact_hash": "21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5", "away_team": "Bread Eaters Esports", "event_id": "156609", "event_start_utc": "2026-10-14T10:30:00Z", "features": {"away_elo": 1498.749903, "away_history_count": 4, "home_elo": 1535.88104, "home_history_count": 34}, "historical_source_observation_times_verified": false, "home_team": "EAC Extra", "inference_inputs": {"book_state": {"games_played": {"bo3:1:25008": 34, "bo3:1:25395": 4}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 40.0, "last_match_utc": {"bo3:1:25008": "2026-10-10T10:30:00Z", "bo3:1:25395": "2026-10-12T08:25:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.06816528215678655, "platt_slope": 0.8746273142827576, "ratings": {"bo3:1:25008": 1535.88104, "bo3:1:25395": 1498.749903}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "8d25951d04320147b4f82f35408c7948ac3d6a80af203ada3bac1aa630e7b330", "features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872"}, "reference_date": "2026-10-13T22:29:07.911078+00:00", "team_ids": ["bo3:1:25008", "bo3:1:25395"]}, "market_type": "moneyline", "model_version": "cs2-tiered-elo-v6", "observed_at_utc": "2026-10-13T22:29:07.911078+00:00", "probabilities": {"away": 0.46316, "home": 0.53684}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "56dd270c1fd3df54f8bd37261678a756b5935a486d91d2a42dbe362cef93c2be", "sport": "CS2"}</t>
+          <t>{"artifact_hash": "642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7", "away_team": "6666", "event_id": "156908", "event_start_utc": "2026-10-14T11:00:00Z", "features": {"away_elo": 1681.920979, "away_history_count": 38, "home_elo": 1522.414525, "home_history_count": 187}, "historical_source_observation_times_verified": false, "home_team": "los kogutos", "inference_inputs": {"book_state": {"games_played": {"bo3:1:1093": 187, "bo3:1:24507": 38}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 40.0, "last_match_utc": {"bo3:1:1093": "2026-10-11T16:25:00Z", "bo3:1:24507": "2026-10-13T17:00:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.06821870672347567, "platt_slope": 0.8748911450799665, "ratings": {"bo3:1:1093": 1522.414525, "bo3:1:24507": 1681.920979}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "3abbfc5d7124cc94603dada2e4c996da231a679d437c5a066d994a2a7d428f61", "features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872"}, "reference_date": "2026-10-14T05:52:14.154858+00:00", "team_ids": ["bo3:1:1093", "bo3:1:24507"]}, "market_type": "moneyline", "model_version": "cs2-tiered-elo-v6", "observed_at_utc": "2026-10-14T05:52:14.154858+00:00", "probabilities": {"away": 0.650526, "home": 0.349474}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "e1736e366ffc3e00b5d6423d98fb7909dc379218ce145d44ac462a20927b9191", "sport": "CS2"}</t>
         </is>
       </c>
     </row>
     <row r="139" ht="36" customHeight="1">
       <c r="A139" s="24" t="inlineStr">
         <is>
-          <t>104afc50657c409e</t>
+          <t>cffb6e478af441b4</t>
         </is>
       </c>
       <c r="B139" s="24" t="inlineStr">
         <is>
-          <t>2026-10-13T22:38:44.831854Z</t>
+          <t>2026-10-14T06:03:43.455911Z</t>
         </is>
       </c>
       <c r="C139" s="24" t="inlineStr">
@@ -45420,7 +45420,7 @@
       </c>
       <c r="D139" s="24" t="inlineStr">
         <is>
-          <t>157862</t>
+          <t>157359</t>
         </is>
       </c>
       <c r="E139" s="24" t="inlineStr">
@@ -45430,12 +45430,12 @@
       </c>
       <c r="F139" s="24" t="inlineStr">
         <is>
-          <t>BakS eSports</t>
+          <t>mellren</t>
         </is>
       </c>
       <c r="G139" s="24" t="inlineStr">
         <is>
-          <t>Bushido Wildcats</t>
+          <t>ex-RUSTEC</t>
         </is>
       </c>
       <c r="H139" s="24" t="inlineStr">
@@ -45445,7 +45445,7 @@
       </c>
       <c r="I139" s="24" t="inlineStr">
         <is>
-          <t>away</t>
+          <t>home</t>
         </is>
       </c>
       <c r="J139" s="25" t="n"/>
@@ -45455,20 +45455,20 @@
         </is>
       </c>
       <c r="L139" s="26" t="n">
-        <v>-144</v>
+        <v>-194</v>
       </c>
       <c r="M139" s="27" t="n">
-        <v>1.694444</v>
+        <v>1.515464</v>
       </c>
       <c r="N139" s="28" t="n">
-        <v>0.590164</v>
+        <v>0.659864</v>
       </c>
       <c r="O139" s="28" t="n">
-        <v>0.549037</v>
+        <v>0.609986</v>
       </c>
       <c r="P139" s="28" t="n"/>
       <c r="Q139" s="28" t="n">
-        <v>-0.041127</v>
+        <v>-0.049878</v>
       </c>
       <c r="R139" s="26" t="n">
         <v>0</v>
@@ -45497,7 +45497,7 @@
       <c r="AD139" s="24" t="n"/>
       <c r="AE139" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.5900 (market_slug=aec-cs2-bw-baks-2026-10-14).</t>
+          <t>Neutral Elo baseline; executable ask 0.6600 (market_slug=aec-cs2-erx-mel-2026-10-14).</t>
         </is>
       </c>
       <c r="AF139" s="31" t="inlineStr">
@@ -45538,32 +45538,32 @@
       </c>
       <c r="AP139" s="24" t="inlineStr">
         <is>
-          <t>BakS eSports</t>
+          <t>mellren</t>
         </is>
       </c>
       <c r="AQ139" s="24" t="inlineStr">
         <is>
-          <t>BakS eSports</t>
+          <t>mellren</t>
         </is>
       </c>
       <c r="AR139" s="24" t="inlineStr">
         <is>
-          <t>BakS eSports</t>
+          <t>mellren</t>
         </is>
       </c>
       <c r="AS139" s="24" t="inlineStr">
         <is>
-          <t>Bushido Wildcats</t>
+          <t>ex-RUSTEC</t>
         </is>
       </c>
       <c r="AT139" s="24" t="inlineStr">
         <is>
-          <t>Bushido Wildcats</t>
+          <t>ex-RUSTEC</t>
         </is>
       </c>
       <c r="AU139" s="24" t="inlineStr">
         <is>
-          <t>Bushido Wildcats</t>
+          <t>ex-RUSTEC</t>
         </is>
       </c>
       <c r="AV139" s="24" t="n"/>
@@ -45581,7 +45581,7 @@
       </c>
       <c r="BA139" s="24" t="inlineStr">
         <is>
-          <t>21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5</t>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
         </is>
       </c>
       <c r="BB139" s="24" t="inlineStr">
@@ -45596,7 +45596,7 @@
       </c>
       <c r="BD139" s="24" t="inlineStr">
         <is>
-          <t>21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5</t>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
         </is>
       </c>
       <c r="BE139" s="24" t="inlineStr">
@@ -45616,7 +45616,7 @@
       </c>
       <c r="BH139" s="24" t="inlineStr">
         <is>
-          <t>2026-10-13T22:34:46.609615Z</t>
+          <t>2026-10-14T05:57:56.537626Z</t>
         </is>
       </c>
       <c r="BI139" s="24" t="inlineStr">
@@ -45626,13 +45626,13 @@
       </c>
       <c r="BJ139" s="25" t="n"/>
       <c r="BK139" s="26" t="n">
-        <v>-144</v>
+        <v>-194</v>
       </c>
       <c r="BL139" s="27" t="n">
-        <v>1.694444</v>
+        <v>1.515464</v>
       </c>
       <c r="BM139" s="28" t="n">
-        <v>0.590164</v>
+        <v>0.659864</v>
       </c>
       <c r="BN139" s="28" t="n"/>
       <c r="BO139" s="28" t="n"/>
@@ -45695,29 +45695,29 @@
       <c r="DP139" s="24" t="n"/>
       <c r="DQ139" s="24" t="inlineStr">
         <is>
-          <t>{"artifact_hash": "21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5", "away_team": "BakS eSports", "event_id": "157862", "event_start_utc": "2026-10-14T11:00:00Z", "features": {"away_elo": 1652.176773, "away_history_count": 166, "home_elo": 1592.079131, "home_history_count": 219}, "historical_source_observation_times_verified": false, "home_team": "Bushido Wildcats", "inference_inputs": {"book_state": {"games_played": {"bo3:1:20792": 219, "bo3:1:2924": 166}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 40.0, "last_match_utc": {"bo3:1:20792": "2026-10-13T11:00:00Z", "bo3:1:2924": "2026-10-13T08:00:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.06816528215678655, "platt_slope": 0.8746273142827576, "ratings": {"bo3:1:20792": 1592.079131, "bo3:1:2924": 1652.176773}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "8d25951d04320147b4f82f35408c7948ac3d6a80af203ada3bac1aa630e7b330", "features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872"}, "reference_date": "2026-10-13T22:29:07.911078+00:00", "team_ids": ["bo3:1:20792", "bo3:1:2924"]}, "market_type": "moneyline", "model_version": "cs2-tiered-elo-v6", "observed_at_utc": "2026-10-13T22:29:07.911078+00:00", "probabilities": {"away": 0.549037, "home": 0.450963}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "86d9af3bc2dd331e3245b1f031ec2824a457f6ce219f0091419f58e2228fae8c", "sport": "CS2"}</t>
+          <t>{"artifact_hash": "642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7", "away_team": "mellren", "event_id": "157359", "event_start_utc": "2026-10-14T11:00:00Z", "features": {"away_elo": 1695.569989, "away_history_count": 56, "home_elo": 1787.204398, "home_history_count": 64}, "historical_source_observation_times_verified": false, "home_team": "ex-RUSTEC", "inference_inputs": {"book_state": {"games_played": {"bo3:1:23102": 56, "bo3:1:24857": 64}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 40.0, "last_match_utc": {"bo3:1:23102": "2026-10-12T11:10:00Z", "bo3:1:24857": "2026-10-12T21:20:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.06821870672347567, "platt_slope": 0.8748911450799665, "ratings": {"bo3:1:23102": 1695.569989, "bo3:1:24857": 1787.204398}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "3abbfc5d7124cc94603dada2e4c996da231a679d437c5a066d994a2a7d428f61", "features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872"}, "reference_date": "2026-10-14T05:52:14.154858+00:00", "team_ids": ["bo3:1:24857", "bo3:1:23102"]}, "market_type": "moneyline", "model_version": "cs2-tiered-elo-v6", "observed_at_utc": "2026-10-14T05:52:14.154858+00:00", "probabilities": {"away": 0.390014, "home": 0.609986}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "4cbaf57b6ec7114bf681f7b0ef94c1cbed7612634d1e05303e00b03b3e427663", "sport": "CS2"}</t>
         </is>
       </c>
     </row>
     <row r="140" ht="36" customHeight="1">
       <c r="A140" s="24" t="inlineStr">
         <is>
-          <t>02000aa5b9fd4818</t>
+          <t>6ed753a3ef414818</t>
         </is>
       </c>
       <c r="B140" s="24" t="inlineStr">
         <is>
-          <t>2026-10-13T22:38:44.831854Z</t>
+          <t>2026-10-14T06:03:43.455911Z</t>
         </is>
       </c>
       <c r="C140" s="24" t="inlineStr">
         <is>
-          <t>2026-10-14T13:00:00Z</t>
+          <t>2026-10-14T13:30:00Z</t>
         </is>
       </c>
       <c r="D140" s="24" t="inlineStr">
         <is>
-          <t>157272</t>
+          <t>154784</t>
         </is>
       </c>
       <c r="E140" s="24" t="inlineStr">
@@ -45727,55 +45727,57 @@
       </c>
       <c r="F140" s="24" t="inlineStr">
         <is>
-          <t>realgotis22</t>
+          <t>PARIVISION</t>
         </is>
       </c>
       <c r="G140" s="24" t="inlineStr">
         <is>
-          <t>Blitzkrieg</t>
+          <t>Legacy</t>
         </is>
       </c>
       <c r="H140" s="24" t="inlineStr">
         <is>
-          <t>moneyline</t>
+          <t>total</t>
         </is>
       </c>
       <c r="I140" s="24" t="inlineStr">
         <is>
-          <t>away</t>
-        </is>
-      </c>
-      <c r="J140" s="25" t="n"/>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="J140" s="25" t="n">
+        <v>2.5</v>
+      </c>
       <c r="K140" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
         </is>
       </c>
       <c r="L140" s="26" t="n">
-        <v>-122</v>
+        <v>-133</v>
       </c>
       <c r="M140" s="27" t="n">
-        <v>1.819672</v>
+        <v>1.75188</v>
       </c>
       <c r="N140" s="28" t="n">
-        <v>0.54955</v>
+        <v>0.570815</v>
       </c>
       <c r="O140" s="28" t="n">
-        <v>0.657821</v>
+        <v>0.503866</v>
       </c>
       <c r="P140" s="28" t="n"/>
       <c r="Q140" s="28" t="n">
-        <v>0.108271</v>
+        <v>-0.06694899999999999</v>
       </c>
       <c r="R140" s="26" t="n">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="S140" s="29" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="T140" s="24" t="inlineStr">
         <is>
-          <t>cs2-tiered-elo-v6</t>
+          <t>cs2-total-tiered-elo-v6</t>
         </is>
       </c>
       <c r="U140" s="24" t="inlineStr">
@@ -45794,7 +45796,7 @@
       <c r="AD140" s="24" t="n"/>
       <c r="AE140" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.5500 (market_slug=aec-cs2-bk-rea-2026-10-14).</t>
+          <t>Neutral Elo baseline; executable ask 0.5700 (market_slug=tsc-cs2-lgc-prv-2026-10-14-tot-2pt5).</t>
         </is>
       </c>
       <c r="AF140" s="31" t="inlineStr">
@@ -45812,7 +45814,7 @@
       <c r="AJ140" s="31" t="n"/>
       <c r="AK140" s="24" t="inlineStr">
         <is>
-          <t>model_qualified</t>
+          <t>paper_call</t>
         </is>
       </c>
       <c r="AL140" s="26" t="n">
@@ -45820,7 +45822,7 @@
       </c>
       <c r="AM140" s="24" t="inlineStr">
         <is>
-          <t>QUALIFIED_SHADOW_CALL</t>
+          <t>RESEARCH_OBSERVATION</t>
         </is>
       </c>
       <c r="AN140" s="24" t="inlineStr">
@@ -45830,37 +45832,37 @@
       </c>
       <c r="AO140" s="24" t="inlineStr">
         <is>
-          <t>QUALIFIED</t>
+          <t>PAPER_CALL_LOW_EDGE</t>
         </is>
       </c>
       <c r="AP140" s="24" t="inlineStr">
         <is>
-          <t>realgotis22</t>
+          <t>PARIVISION</t>
         </is>
       </c>
       <c r="AQ140" s="24" t="inlineStr">
         <is>
-          <t>realgotis22</t>
+          <t>PARIVISION</t>
         </is>
       </c>
       <c r="AR140" s="24" t="inlineStr">
         <is>
-          <t>realgotis22</t>
+          <t>PARIVISION</t>
         </is>
       </c>
       <c r="AS140" s="24" t="inlineStr">
         <is>
-          <t>Blitzkrieg</t>
+          <t>Legacy</t>
         </is>
       </c>
       <c r="AT140" s="24" t="inlineStr">
         <is>
-          <t>Blitzkrieg</t>
+          <t>Legacy</t>
         </is>
       </c>
       <c r="AU140" s="24" t="inlineStr">
         <is>
-          <t>Blitzkrieg</t>
+          <t>Legacy</t>
         </is>
       </c>
       <c r="AV140" s="24" t="n"/>
@@ -45878,7 +45880,7 @@
       </c>
       <c r="BA140" s="24" t="inlineStr">
         <is>
-          <t>21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5</t>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
         </is>
       </c>
       <c r="BB140" s="24" t="inlineStr">
@@ -45888,12 +45890,12 @@
       </c>
       <c r="BC140" s="24" t="inlineStr">
         <is>
-          <t>cs2-tiered-elo-v6</t>
+          <t>cs2-total-tiered-elo-v6</t>
         </is>
       </c>
       <c r="BD140" s="24" t="inlineStr">
         <is>
-          <t>21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5</t>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
         </is>
       </c>
       <c r="BE140" s="24" t="inlineStr">
@@ -45908,12 +45910,12 @@
       </c>
       <c r="BG140" s="24" t="inlineStr">
         <is>
-          <t>cs2-tiered-elo-v6</t>
+          <t>cs2-total-tiered-elo-v6</t>
         </is>
       </c>
       <c r="BH140" s="24" t="inlineStr">
         <is>
-          <t>2026-10-13T22:34:56.975938Z</t>
+          <t>2026-10-14T05:59:08.842775Z</t>
         </is>
       </c>
       <c r="BI140" s="24" t="inlineStr">
@@ -45921,15 +45923,17 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ140" s="25" t="n"/>
+      <c r="BJ140" s="25" t="n">
+        <v>2.5</v>
+      </c>
       <c r="BK140" s="26" t="n">
-        <v>-122</v>
+        <v>-133</v>
       </c>
       <c r="BL140" s="27" t="n">
-        <v>1.819672</v>
+        <v>1.75188</v>
       </c>
       <c r="BM140" s="28" t="n">
-        <v>0.54955</v>
+        <v>0.570815</v>
       </c>
       <c r="BN140" s="28" t="n"/>
       <c r="BO140" s="28" t="n"/>
@@ -45964,7 +45968,7 @@
       <c r="CR140" s="24" t="n"/>
       <c r="CS140" s="24" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
       <c r="CT140" s="24" t="n"/>
@@ -45990,31 +45994,27 @@
       <c r="DN140" s="24" t="n"/>
       <c r="DO140" s="24" t="n"/>
       <c r="DP140" s="24" t="n"/>
-      <c r="DQ140" s="24" t="inlineStr">
-        <is>
-          <t>{"artifact_hash": "21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5", "away_team": "realgotis22", "event_id": "157272", "event_start_utc": "2026-10-14T13:00:00Z", "features": {"away_elo": 1628.485971, "away_history_count": 189, "home_elo": 1350.457607, "home_history_count": 13}, "historical_source_observation_times_verified": false, "home_team": "Blitzkrieg", "inference_inputs": {"book_state": {"games_played": {"bo3:1:19951": 189, "bo3:1:4264": 13}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 40.0, "last_match_utc": {"bo3:1:19951": "2026-05-30T14:00:00Z", "bo3:1:4264": "2026-08-31T16:00:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.06816528215678655, "platt_slope": 0.8746273142827576, "ratings": {"bo3:1:19951": 1628.485971, "bo3:1:4264": 1350.457607}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "8d25951d04320147b4f82f35408c7948ac3d6a80af203ada3bac1aa630e7b330", "features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872"}, "reference_date": "2026-10-13T22:29:07.911078+00:00", "team_ids": ["bo3:1:4264", "bo3:1:19951"]}, "market_type": "moneyline", "model_version": "cs2-tiered-elo-v6", "observed_at_utc": "2026-10-13T22:29:07.911078+00:00", "probabilities": {"away": 0.657821, "home": 0.342179}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "96206caafeb8fd7823a208a1c38ccd1230f1dbb4324e22527e42bb1c9af7bac8", "sport": "CS2"}</t>
-        </is>
-      </c>
+      <c r="DQ140" s="24" t="n"/>
     </row>
     <row r="141" ht="36" customHeight="1">
       <c r="A141" s="24" t="inlineStr">
         <is>
-          <t>f8eb609698c84305</t>
+          <t>cafa0bb254554486</t>
         </is>
       </c>
       <c r="B141" s="24" t="inlineStr">
         <is>
-          <t>2026-10-13T22:38:44.831854Z</t>
+          <t>2026-10-14T06:03:43.455911Z</t>
         </is>
       </c>
       <c r="C141" s="24" t="inlineStr">
         <is>
-          <t>2026-10-14T13:30:00Z</t>
+          <t>2026-10-14T14:00:00Z</t>
         </is>
       </c>
       <c r="D141" s="24" t="inlineStr">
         <is>
-          <t>154784</t>
+          <t>157863</t>
         </is>
       </c>
       <c r="E141" s="24" t="inlineStr">
@@ -46024,12 +46024,12 @@
       </c>
       <c r="F141" s="24" t="inlineStr">
         <is>
-          <t>PARIVISION</t>
+          <t>FORZE Reload</t>
         </is>
       </c>
       <c r="G141" s="24" t="inlineStr">
         <is>
-          <t>Legacy</t>
+          <t>BET-M 33</t>
         </is>
       </c>
       <c r="H141" s="24" t="inlineStr">
@@ -46049,23 +46049,23 @@
         </is>
       </c>
       <c r="L141" s="26" t="n">
-        <v>-144</v>
+        <v>-117</v>
       </c>
       <c r="M141" s="27" t="n">
-        <v>1.694444</v>
+        <v>1.854701</v>
       </c>
       <c r="N141" s="28" t="n">
-        <v>0.590164</v>
+        <v>0.539171</v>
       </c>
       <c r="O141" s="28" t="n">
-        <v>0.565879</v>
+        <v>0.590184</v>
       </c>
       <c r="P141" s="28" t="n"/>
       <c r="Q141" s="28" t="n">
-        <v>-0.024285</v>
+        <v>0.051013</v>
       </c>
       <c r="R141" s="26" t="n">
-        <v>8</v>
+        <v>46</v>
       </c>
       <c r="S141" s="29" t="n">
         <v>1</v>
@@ -46091,7 +46091,7 @@
       <c r="AD141" s="24" t="n"/>
       <c r="AE141" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.5900 (market_slug=aec-cs2-lgc-prv-2026-10-14).</t>
+          <t>Neutral Elo baseline; executable ask 0.5400 (market_slug=aec-cs2-33-forzer-2026-10-14).</t>
         </is>
       </c>
       <c r="AF141" s="31" t="inlineStr">
@@ -46109,7 +46109,7 @@
       <c r="AJ141" s="31" t="n"/>
       <c r="AK141" s="24" t="inlineStr">
         <is>
-          <t>paper_call</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL141" s="26" t="n">
@@ -46117,7 +46117,7 @@
       </c>
       <c r="AM141" s="24" t="inlineStr">
         <is>
-          <t>RESEARCH_OBSERVATION</t>
+          <t>QUALIFIED_SHADOW_CALL</t>
         </is>
       </c>
       <c r="AN141" s="24" t="inlineStr">
@@ -46127,37 +46127,37 @@
       </c>
       <c r="AO141" s="24" t="inlineStr">
         <is>
-          <t>PAPER_CALL_LOW_EDGE</t>
+          <t>QUALIFIED</t>
         </is>
       </c>
       <c r="AP141" s="24" t="inlineStr">
         <is>
-          <t>PARIVISION</t>
+          <t>FORZE Reload</t>
         </is>
       </c>
       <c r="AQ141" s="24" t="inlineStr">
         <is>
-          <t>PARIVISION</t>
+          <t>FORZE Reload</t>
         </is>
       </c>
       <c r="AR141" s="24" t="inlineStr">
         <is>
-          <t>PARIVISION</t>
+          <t>FORZE Reload</t>
         </is>
       </c>
       <c r="AS141" s="24" t="inlineStr">
         <is>
-          <t>Legacy</t>
+          <t>BET-M 33</t>
         </is>
       </c>
       <c r="AT141" s="24" t="inlineStr">
         <is>
-          <t>Legacy</t>
+          <t>BET-M 33</t>
         </is>
       </c>
       <c r="AU141" s="24" t="inlineStr">
         <is>
-          <t>Legacy</t>
+          <t>BET-M 33</t>
         </is>
       </c>
       <c r="AV141" s="24" t="n"/>
@@ -46175,7 +46175,7 @@
       </c>
       <c r="BA141" s="24" t="inlineStr">
         <is>
-          <t>21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5</t>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
         </is>
       </c>
       <c r="BB141" s="24" t="inlineStr">
@@ -46190,7 +46190,7 @@
       </c>
       <c r="BD141" s="24" t="inlineStr">
         <is>
-          <t>21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5</t>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
         </is>
       </c>
       <c r="BE141" s="24" t="inlineStr">
@@ -46210,7 +46210,7 @@
       </c>
       <c r="BH141" s="24" t="inlineStr">
         <is>
-          <t>2026-10-13T22:35:17.807103Z</t>
+          <t>2026-10-14T05:59:50.745423Z</t>
         </is>
       </c>
       <c r="BI141" s="24" t="inlineStr">
@@ -46220,13 +46220,13 @@
       </c>
       <c r="BJ141" s="25" t="n"/>
       <c r="BK141" s="26" t="n">
-        <v>-144</v>
+        <v>-117</v>
       </c>
       <c r="BL141" s="27" t="n">
-        <v>1.694444</v>
+        <v>1.854701</v>
       </c>
       <c r="BM141" s="28" t="n">
-        <v>0.590164</v>
+        <v>0.539171</v>
       </c>
       <c r="BN141" s="28" t="n"/>
       <c r="BO141" s="28" t="n"/>
@@ -46261,7 +46261,7 @@
       <c r="CR141" s="24" t="n"/>
       <c r="CS141" s="24" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="CT141" s="24" t="n"/>
@@ -46289,19 +46289,19 @@
       <c r="DP141" s="24" t="n"/>
       <c r="DQ141" s="24" t="inlineStr">
         <is>
-          <t>{"artifact_hash": "21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5", "away_team": "PARIVISION", "event_id": "154784", "event_start_utc": "2026-10-14T13:30:00Z", "features": {"away_elo": 1996.647414, "away_history_count": 297, "home_elo": 2060.918049, "home_history_count": 304}, "historical_source_observation_times_verified": false, "home_team": "Legacy", "inference_inputs": {"book_state": {"games_played": {"bo3:1:8118": 304, "bo3:1:8171": 297}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 40.0, "last_match_utc": {"bo3:1:8118": "2026-10-06T17:00:00Z", "bo3:1:8171": "2026-10-09T11:30:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.06816528215678655, "platt_slope": 0.8746273142827576, "ratings": {"bo3:1:8118": 2060.918049, "bo3:1:8171": 1996.647414}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "8d25951d04320147b4f82f35408c7948ac3d6a80af203ada3bac1aa630e7b330", "features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872"}, "reference_date": "2026-10-13T22:29:07.911078+00:00", "team_ids": ["bo3:1:8118", "bo3:1:8171"]}, "market_type": "moneyline", "model_version": "cs2-tiered-elo-v6", "observed_at_utc": "2026-10-13T22:29:07.911078+00:00", "probabilities": {"away": 0.434121, "home": 0.565879}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "4ab4fd1a006265997209ae11a027a1ebac7bd1799e2204b07d48ce6c6ac970fe", "sport": "CS2"}</t>
+          <t>{"artifact_hash": "642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7", "away_team": "FORZE Reload", "event_id": "157863", "event_start_utc": "2026-10-14T14:00:00Z", "features": {"away_elo": 1675.326686, "away_history_count": 332, "home_elo": 1738.15062, "home_history_count": 178}, "historical_source_observation_times_verified": false, "home_team": "BET-M 33", "inference_inputs": {"book_state": {"games_played": {"bo3:1:10703": 332, "bo3:1:22191": 178}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 40.0, "last_match_utc": {"bo3:1:10703": "2026-10-04T13:45:00Z", "bo3:1:22191": "2026-10-11T17:00:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.06821870672347567, "platt_slope": 0.8748911450799665, "ratings": {"bo3:1:10703": 1675.326686, "bo3:1:22191": 1738.15062}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "3abbfc5d7124cc94603dada2e4c996da231a679d437c5a066d994a2a7d428f61", "features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872"}, "reference_date": "2026-10-14T05:52:14.154858+00:00", "team_ids": ["bo3:1:22191", "bo3:1:10703"]}, "market_type": "moneyline", "model_version": "cs2-tiered-elo-v6", "observed_at_utc": "2026-10-14T05:52:14.154858+00:00", "probabilities": {"away": 0.409816, "home": 0.590184}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "bbe81590e925cd7635614102892849d3282466b446d883131b13c185b4483323", "sport": "CS2"}</t>
         </is>
       </c>
     </row>
     <row r="142" ht="36" customHeight="1">
       <c r="A142" s="24" t="inlineStr">
         <is>
-          <t>6030bb278aaf437f</t>
+          <t>4ed85e5b665c4664</t>
         </is>
       </c>
       <c r="B142" s="24" t="inlineStr">
         <is>
-          <t>2026-10-13T22:38:44.831854Z</t>
+          <t>2026-10-14T06:03:43.455911Z</t>
         </is>
       </c>
       <c r="C142" s="24" t="inlineStr">
@@ -46311,7 +46311,7 @@
       </c>
       <c r="D142" s="24" t="inlineStr">
         <is>
-          <t>157360</t>
+          <t>159046</t>
         </is>
       </c>
       <c r="E142" s="24" t="inlineStr">
@@ -46321,12 +46321,12 @@
       </c>
       <c r="F142" s="24" t="inlineStr">
         <is>
-          <t>The Last Resort</t>
+          <t>UPGRADE</t>
         </is>
       </c>
       <c r="G142" s="24" t="inlineStr">
         <is>
-          <t>G2 Ares</t>
+          <t>Butterfly</t>
         </is>
       </c>
       <c r="H142" s="24" t="inlineStr">
@@ -46346,26 +46346,26 @@
         </is>
       </c>
       <c r="L142" s="26" t="n">
-        <v>-213</v>
+        <v>-108</v>
       </c>
       <c r="M142" s="27" t="n">
-        <v>1.469484</v>
+        <v>1.925926</v>
       </c>
       <c r="N142" s="28" t="n">
-        <v>0.680511</v>
+        <v>0.519231</v>
       </c>
       <c r="O142" s="28" t="n">
-        <v>0.628134</v>
+        <v>0.637364</v>
       </c>
       <c r="P142" s="28" t="n"/>
       <c r="Q142" s="28" t="n">
-        <v>-0.052377</v>
+        <v>0.118133</v>
       </c>
       <c r="R142" s="26" t="n">
-        <v>0</v>
+        <v>79</v>
       </c>
       <c r="S142" s="29" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="T142" s="24" t="inlineStr">
         <is>
@@ -46388,7 +46388,7 @@
       <c r="AD142" s="24" t="n"/>
       <c r="AE142" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.6800 (market_slug=aec-cs2-g2a-tlr-2026-10-14).</t>
+          <t>Neutral Elo baseline; executable ask 0.5200 (market_slug=aec-cs2-btf-upg-2026-10-14).</t>
         </is>
       </c>
       <c r="AF142" s="31" t="inlineStr">
@@ -46406,7 +46406,7 @@
       <c r="AJ142" s="31" t="n"/>
       <c r="AK142" s="24" t="inlineStr">
         <is>
-          <t>paper_call</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL142" s="26" t="n">
@@ -46414,7 +46414,7 @@
       </c>
       <c r="AM142" s="24" t="inlineStr">
         <is>
-          <t>RESEARCH_OBSERVATION</t>
+          <t>QUALIFIED_SHADOW_CALL</t>
         </is>
       </c>
       <c r="AN142" s="24" t="inlineStr">
@@ -46424,37 +46424,37 @@
       </c>
       <c r="AO142" s="24" t="inlineStr">
         <is>
-          <t>PAPER_CALL_LOW_EDGE</t>
+          <t>QUALIFIED</t>
         </is>
       </c>
       <c r="AP142" s="24" t="inlineStr">
         <is>
-          <t>The Last Resort</t>
+          <t>UPGRADE</t>
         </is>
       </c>
       <c r="AQ142" s="24" t="inlineStr">
         <is>
-          <t>The Last Resort</t>
+          <t>UPGRADE</t>
         </is>
       </c>
       <c r="AR142" s="24" t="inlineStr">
         <is>
-          <t>The Last Resort</t>
+          <t>UPGRADE</t>
         </is>
       </c>
       <c r="AS142" s="24" t="inlineStr">
         <is>
-          <t>G2 Ares</t>
+          <t>Butterfly</t>
         </is>
       </c>
       <c r="AT142" s="24" t="inlineStr">
         <is>
-          <t>G2 Ares</t>
+          <t>Butterfly</t>
         </is>
       </c>
       <c r="AU142" s="24" t="inlineStr">
         <is>
-          <t>G2 Ares</t>
+          <t>Butterfly</t>
         </is>
       </c>
       <c r="AV142" s="24" t="n"/>
@@ -46472,7 +46472,7 @@
       </c>
       <c r="BA142" s="24" t="inlineStr">
         <is>
-          <t>21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5</t>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
         </is>
       </c>
       <c r="BB142" s="24" t="inlineStr">
@@ -46487,7 +46487,7 @@
       </c>
       <c r="BD142" s="24" t="inlineStr">
         <is>
-          <t>21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5</t>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
         </is>
       </c>
       <c r="BE142" s="24" t="inlineStr">
@@ -46507,7 +46507,7 @@
       </c>
       <c r="BH142" s="24" t="inlineStr">
         <is>
-          <t>2026-10-13T22:35:49.210423Z</t>
+          <t>2026-10-14T06:00:22.148335Z</t>
         </is>
       </c>
       <c r="BI142" s="24" t="inlineStr">
@@ -46517,13 +46517,13 @@
       </c>
       <c r="BJ142" s="25" t="n"/>
       <c r="BK142" s="26" t="n">
-        <v>-213</v>
+        <v>-108</v>
       </c>
       <c r="BL142" s="27" t="n">
-        <v>1.469484</v>
+        <v>1.925926</v>
       </c>
       <c r="BM142" s="28" t="n">
-        <v>0.680511</v>
+        <v>0.519231</v>
       </c>
       <c r="BN142" s="28" t="n"/>
       <c r="BO142" s="28" t="n"/>
@@ -46558,7 +46558,7 @@
       <c r="CR142" s="24" t="n"/>
       <c r="CS142" s="24" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="CT142" s="24" t="n"/>
@@ -46586,29 +46586,29 @@
       <c r="DP142" s="24" t="n"/>
       <c r="DQ142" s="24" t="inlineStr">
         <is>
-          <t>{"artifact_hash": "21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5", "away_team": "The Last Resort", "event_id": "157360", "event_start_utc": "2026-10-14T14:00:00Z", "features": {"away_elo": 1467.951929, "away_history_count": 147, "home_elo": 1581.891651, "home_history_count": 284}, "historical_source_observation_times_verified": false, "home_team": "G2 Ares", "inference_inputs": {"book_state": {"games_played": {"bo3:1:10994": 284, "bo3:1:2740": 147}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 40.0, "last_match_utc": {"bo3:1:10994": "2026-10-09T17:30:00Z", "bo3:1:2740": "2026-10-08T13:00:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.06816528215678655, "platt_slope": 0.8746273142827576, "ratings": {"bo3:1:10994": 1581.891651, "bo3:1:2740": 1467.951929}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "8d25951d04320147b4f82f35408c7948ac3d6a80af203ada3bac1aa630e7b330", "features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872"}, "reference_date": "2026-10-13T22:29:07.911078+00:00", "team_ids": ["bo3:1:10994", "bo3:1:2740"]}, "market_type": "moneyline", "model_version": "cs2-tiered-elo-v6", "observed_at_utc": "2026-10-13T22:29:07.911078+00:00", "probabilities": {"away": 0.371866, "home": 0.628134}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "d2d9af04aa717b805d4231f3c9c722536fd672d7b88ccef6f0358a42302473cb", "sport": "CS2"}</t>
+          <t>{"artifact_hash": "642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7", "away_team": "UPGRADE", "event_id": "159046", "event_start_utc": "2026-10-14T14:00:00Z", "features": {"away_elo": 1537.218061, "away_history_count": 11, "home_elo": 1660.985544, "home_history_count": 30}, "historical_source_observation_times_verified": false, "home_team": "Butterfly", "inference_inputs": {"book_state": {"games_played": {"bo3:1:24855": 30, "bo3:1:25212": 11}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 40.0, "last_match_utc": {"bo3:1:24855": "2026-10-06T14:00:00Z", "bo3:1:25212": "2026-09-25T14:45:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.06821870672347567, "platt_slope": 0.8748911450799665, "ratings": {"bo3:1:24855": 1660.985544, "bo3:1:25212": 1537.218061}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "3abbfc5d7124cc94603dada2e4c996da231a679d437c5a066d994a2a7d428f61", "features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872"}, "reference_date": "2026-10-14T05:52:14.154858+00:00", "team_ids": ["bo3:1:24855", "bo3:1:25212"]}, "market_type": "moneyline", "model_version": "cs2-tiered-elo-v6", "observed_at_utc": "2026-10-14T05:52:14.154858+00:00", "probabilities": {"away": 0.362636, "home": 0.637364}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "b7e859df509a56ba4bda50a559c47f8c4d8d4cfd98d4b4f89bf0e069551b98bd", "sport": "CS2"}</t>
         </is>
       </c>
     </row>
     <row r="143" ht="36" customHeight="1">
       <c r="A143" s="24" t="inlineStr">
         <is>
-          <t>d06438201f774c06</t>
+          <t>b18eb4bd053343ef</t>
         </is>
       </c>
       <c r="B143" s="24" t="inlineStr">
         <is>
-          <t>2026-10-13T22:38:44.831854Z</t>
+          <t>2026-10-14T06:03:43.455911Z</t>
         </is>
       </c>
       <c r="C143" s="24" t="inlineStr">
         <is>
-          <t>2026-10-14T16:00:00Z</t>
+          <t>2026-10-14T14:00:00Z</t>
         </is>
       </c>
       <c r="D143" s="24" t="inlineStr">
         <is>
-          <t>154958</t>
+          <t>159047</t>
         </is>
       </c>
       <c r="E143" s="24" t="inlineStr">
@@ -46618,12 +46618,12 @@
       </c>
       <c r="F143" s="24" t="inlineStr">
         <is>
-          <t>Playing Ducks</t>
+          <t>Phantom</t>
         </is>
       </c>
       <c r="G143" s="24" t="inlineStr">
         <is>
-          <t>Sissi State Punks</t>
+          <t>Nuclear TigeRES</t>
         </is>
       </c>
       <c r="H143" s="24" t="inlineStr">
@@ -46633,7 +46633,7 @@
       </c>
       <c r="I143" s="24" t="inlineStr">
         <is>
-          <t>away</t>
+          <t>home</t>
         </is>
       </c>
       <c r="J143" s="25" t="n"/>
@@ -46643,26 +46643,26 @@
         </is>
       </c>
       <c r="L143" s="26" t="n">
-        <v>117</v>
+        <v>-144</v>
       </c>
       <c r="M143" s="27" t="n">
-        <v>2.17</v>
+        <v>1.694444</v>
       </c>
       <c r="N143" s="28" t="n">
-        <v>0.460829</v>
+        <v>0.590164</v>
       </c>
       <c r="O143" s="28" t="n">
-        <v>0.595395</v>
+        <v>0.6723749999999999</v>
       </c>
       <c r="P143" s="28" t="n"/>
       <c r="Q143" s="28" t="n">
-        <v>0.134566</v>
+        <v>0.08221100000000001</v>
       </c>
       <c r="R143" s="26" t="n">
-        <v>87</v>
+        <v>61</v>
       </c>
       <c r="S143" s="29" t="n">
-        <v>1.5</v>
+        <v>1.25</v>
       </c>
       <c r="T143" s="24" t="inlineStr">
         <is>
@@ -46685,7 +46685,7 @@
       <c r="AD143" s="24" t="n"/>
       <c r="AE143" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.4600 (market_slug=aec-cs2-ssp-ducks-2026-10-14).</t>
+          <t>Neutral Elo baseline; executable ask 0.5900 (market_slug=aec-cs2-ntr-pha-2026-10-14).</t>
         </is>
       </c>
       <c r="AF143" s="31" t="inlineStr">
@@ -46726,32 +46726,32 @@
       </c>
       <c r="AP143" s="24" t="inlineStr">
         <is>
-          <t>Playing Ducks</t>
+          <t>Phantom</t>
         </is>
       </c>
       <c r="AQ143" s="24" t="inlineStr">
         <is>
-          <t>Playing Ducks</t>
+          <t>Phantom</t>
         </is>
       </c>
       <c r="AR143" s="24" t="inlineStr">
         <is>
-          <t>Playing Ducks</t>
+          <t>Phantom</t>
         </is>
       </c>
       <c r="AS143" s="24" t="inlineStr">
         <is>
-          <t>Sissi State Punks</t>
+          <t>Nuclear TigeRES</t>
         </is>
       </c>
       <c r="AT143" s="24" t="inlineStr">
         <is>
-          <t>Sissi State Punks</t>
+          <t>Nuclear TigeRES</t>
         </is>
       </c>
       <c r="AU143" s="24" t="inlineStr">
         <is>
-          <t>Sissi State Punks</t>
+          <t>Nuclear TigeRES</t>
         </is>
       </c>
       <c r="AV143" s="24" t="n"/>
@@ -46769,7 +46769,7 @@
       </c>
       <c r="BA143" s="24" t="inlineStr">
         <is>
-          <t>21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5</t>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
         </is>
       </c>
       <c r="BB143" s="24" t="inlineStr">
@@ -46784,7 +46784,7 @@
       </c>
       <c r="BD143" s="24" t="inlineStr">
         <is>
-          <t>21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5</t>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
         </is>
       </c>
       <c r="BE143" s="24" t="inlineStr">
@@ -46804,7 +46804,7 @@
       </c>
       <c r="BH143" s="24" t="inlineStr">
         <is>
-          <t>2026-10-13T22:37:11.894822Z</t>
+          <t>2026-10-14T06:00:22.422098Z</t>
         </is>
       </c>
       <c r="BI143" s="24" t="inlineStr">
@@ -46814,13 +46814,13 @@
       </c>
       <c r="BJ143" s="25" t="n"/>
       <c r="BK143" s="26" t="n">
-        <v>117</v>
+        <v>-144</v>
       </c>
       <c r="BL143" s="27" t="n">
-        <v>2.17</v>
+        <v>1.694444</v>
       </c>
       <c r="BM143" s="28" t="n">
-        <v>0.460829</v>
+        <v>0.590164</v>
       </c>
       <c r="BN143" s="28" t="n"/>
       <c r="BO143" s="28" t="n"/>
@@ -46883,29 +46883,29 @@
       <c r="DP143" s="24" t="n"/>
       <c r="DQ143" s="24" t="inlineStr">
         <is>
-          <t>{"artifact_hash": "21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5", "away_team": "Playing Ducks", "event_id": "154958", "event_start_utc": "2026-10-14T16:00:00Z", "features": {"away_elo": 1482.311701, "away_history_count": 22, "home_elo": 1362.166392, "home_history_count": 42}, "historical_source_observation_times_verified": false, "home_team": "Sissi State Punks", "inference_inputs": {"book_state": {"games_played": {"bo3:1:1049": 42, "bo3:1:1545": 22}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 40.0, "last_match_utc": {"bo3:1:1049": "2026-09-28T16:15:00Z", "bo3:1:1545": "2026-10-05T18:00:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.06816528215678655, "platt_slope": 0.8746273142827576, "ratings": {"bo3:1:1049": 1362.166392, "bo3:1:1545": 1482.311701}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "8d25951d04320147b4f82f35408c7948ac3d6a80af203ada3bac1aa630e7b330", "features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872"}, "reference_date": "2026-10-13T22:29:07.911078+00:00", "team_ids": ["bo3:1:1049", "bo3:1:1545"]}, "market_type": "moneyline", "model_version": "cs2-tiered-elo-v6", "observed_at_utc": "2026-10-13T22:29:07.911078+00:00", "probabilities": {"away": 0.595395, "home": 0.404605}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "64a480fb303f3297f32b91d352c16164f76cd55bcc9d11a5fb1484a27199d109", "sport": "CS2"}</t>
+          <t>{"artifact_hash": "642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7", "away_team": "Phantom", "event_id": "159047", "event_start_utc": "2026-10-14T14:00:00Z", "features": {"away_elo": 1700.009132, "away_history_count": 199, "home_elo": 1847.589545, "home_history_count": 269}, "historical_source_observation_times_verified": false, "home_team": "Nuclear TigeRES", "inference_inputs": {"book_state": {"games_played": {"bo3:1:18539": 269, "bo3:1:19204": 199}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 40.0, "last_match_utc": {"bo3:1:18539": "2026-10-12T21:20:00Z", "bo3:1:19204": "2026-10-07T15:00:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.06821870672347567, "platt_slope": 0.8748911450799665, "ratings": {"bo3:1:18539": 1847.589545, "bo3:1:19204": 1700.009132}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "3abbfc5d7124cc94603dada2e4c996da231a679d437c5a066d994a2a7d428f61", "features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872"}, "reference_date": "2026-10-14T05:52:14.154858+00:00", "team_ids": ["bo3:1:18539", "bo3:1:19204"]}, "market_type": "moneyline", "model_version": "cs2-tiered-elo-v6", "observed_at_utc": "2026-10-14T05:52:14.154858+00:00", "probabilities": {"away": 0.327625, "home": 0.672375}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "fe57f62671bb64566e68f94aae73fc98b686cd1604a2b7b14a6a5a1e7ecd54e4", "sport": "CS2"}</t>
         </is>
       </c>
     </row>
     <row r="144" ht="36" customHeight="1">
       <c r="A144" s="24" t="inlineStr">
         <is>
-          <t>21d0d1cbcd384776</t>
+          <t>e22f8f82b07a4128</t>
         </is>
       </c>
       <c r="B144" s="24" t="inlineStr">
         <is>
-          <t>2026-10-13T22:38:44.831854Z</t>
+          <t>2026-10-14T06:03:43.455911Z</t>
         </is>
       </c>
       <c r="C144" s="24" t="inlineStr">
         <is>
-          <t>2026-10-14T22:00:00Z</t>
+          <t>2026-10-14T17:00:00Z</t>
         </is>
       </c>
       <c r="D144" s="24" t="inlineStr">
         <is>
-          <t>157275</t>
+          <t>157864</t>
         </is>
       </c>
       <c r="E144" s="24" t="inlineStr">
@@ -46915,12 +46915,12 @@
       </c>
       <c r="F144" s="24" t="inlineStr">
         <is>
-          <t>A NATA</t>
+          <t>ex-RUSTEC</t>
         </is>
       </c>
       <c r="G144" s="24" t="inlineStr">
         <is>
-          <t>Joga de terno</t>
+          <t>Black Phoenix</t>
         </is>
       </c>
       <c r="H144" s="24" t="inlineStr">
@@ -46930,7 +46930,7 @@
       </c>
       <c r="I144" s="24" t="inlineStr">
         <is>
-          <t>away</t>
+          <t>home</t>
         </is>
       </c>
       <c r="J144" s="25" t="n"/>
@@ -46940,26 +46940,26 @@
         </is>
       </c>
       <c r="L144" s="26" t="n">
-        <v>163</v>
+        <v>-186</v>
       </c>
       <c r="M144" s="27" t="n">
-        <v>2.63</v>
+        <v>1.537634</v>
       </c>
       <c r="N144" s="28" t="n">
-        <v>0.380228</v>
+        <v>0.65035</v>
       </c>
       <c r="O144" s="28" t="n">
-        <v>0.51072</v>
+        <v>0.638595</v>
       </c>
       <c r="P144" s="28" t="n"/>
       <c r="Q144" s="28" t="n">
-        <v>0.130492</v>
+        <v>-0.011755</v>
       </c>
       <c r="R144" s="26" t="n">
-        <v>85</v>
+        <v>14</v>
       </c>
       <c r="S144" s="29" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="T144" s="24" t="inlineStr">
         <is>
@@ -46982,7 +46982,7 @@
       <c r="AD144" s="24" t="n"/>
       <c r="AE144" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.3800 (market_slug=aec-cs2-jdt-ana-2026-10-14).</t>
+          <t>Neutral Elo baseline; executable ask 0.6500 (market_slug=aec-cs2-bpl-erx-2026-10-14).</t>
         </is>
       </c>
       <c r="AF144" s="31" t="inlineStr">
@@ -47018,37 +47018,37 @@
       </c>
       <c r="AO144" s="24" t="inlineStr">
         <is>
-          <t>PAPER_CALL_MODEL_UNVALIDATED</t>
+          <t>PAPER_CALL_LOW_EDGE</t>
         </is>
       </c>
       <c r="AP144" s="24" t="inlineStr">
         <is>
-          <t>A NATA</t>
+          <t>ex-RUSTEC</t>
         </is>
       </c>
       <c r="AQ144" s="24" t="inlineStr">
         <is>
-          <t>A NATA</t>
+          <t>ex-RUSTEC</t>
         </is>
       </c>
       <c r="AR144" s="24" t="inlineStr">
         <is>
-          <t>A NATA</t>
+          <t>ex-RUSTEC</t>
         </is>
       </c>
       <c r="AS144" s="24" t="inlineStr">
         <is>
-          <t>Joga de terno</t>
+          <t>Black Phoenix</t>
         </is>
       </c>
       <c r="AT144" s="24" t="inlineStr">
         <is>
-          <t>Joga de terno</t>
+          <t>Black Phoenix</t>
         </is>
       </c>
       <c r="AU144" s="24" t="inlineStr">
         <is>
-          <t>Joga de terno</t>
+          <t>Black Phoenix</t>
         </is>
       </c>
       <c r="AV144" s="24" t="n"/>
@@ -47066,7 +47066,7 @@
       </c>
       <c r="BA144" s="24" t="inlineStr">
         <is>
-          <t>21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5</t>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
         </is>
       </c>
       <c r="BB144" s="24" t="inlineStr">
@@ -47081,7 +47081,7 @@
       </c>
       <c r="BD144" s="24" t="inlineStr">
         <is>
-          <t>21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5</t>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
         </is>
       </c>
       <c r="BE144" s="24" t="inlineStr">
@@ -47101,7 +47101,7 @@
       </c>
       <c r="BH144" s="24" t="inlineStr">
         <is>
-          <t>2026-10-13T22:38:34.462107Z</t>
+          <t>2026-10-14T06:01:57.704728Z</t>
         </is>
       </c>
       <c r="BI144" s="24" t="inlineStr">
@@ -47111,13 +47111,13 @@
       </c>
       <c r="BJ144" s="25" t="n"/>
       <c r="BK144" s="26" t="n">
-        <v>163</v>
+        <v>-186</v>
       </c>
       <c r="BL144" s="27" t="n">
-        <v>2.63</v>
+        <v>1.537634</v>
       </c>
       <c r="BM144" s="28" t="n">
-        <v>0.380228</v>
+        <v>0.65035</v>
       </c>
       <c r="BN144" s="28" t="n"/>
       <c r="BO144" s="28" t="n"/>
@@ -47152,7 +47152,7 @@
       <c r="CR144" s="24" t="n"/>
       <c r="CS144" s="24" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
       <c r="CT144" s="24" t="n"/>
@@ -47180,7 +47180,1789 @@
       <c r="DP144" s="24" t="n"/>
       <c r="DQ144" s="24" t="inlineStr">
         <is>
-          <t>{"artifact_hash": "21a244e029d58075f561215535923b540359cdf781049d520ffd534a32f40de5", "away_team": "A NATA", "event_id": "157275", "event_start_utc": "2026-10-14T22:00:00Z", "features": {"away_elo": 1500.0, "away_history_count": 0, "home_elo": 1415.874603, "home_history_count": 62}, "historical_source_observation_times_verified": false, "home_team": "Joga de terno", "inference_inputs": {"book_state": {"games_played": {"bo3:1:10697": 62}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 40.0, "last_match_utc": {"bo3:1:10697": "2024-12-10T23:00:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.06816528215678655, "platt_slope": 0.8746273142827576, "ratings": {"bo3:1:10697": 1415.874603}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "8d25951d04320147b4f82f35408c7948ac3d6a80af203ada3bac1aa630e7b330", "features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872"}, "reference_date": "2026-10-13T22:29:07.911078+00:00", "team_ids": ["bo3:1:10697", "unknown:anata"]}, "market_type": "moneyline", "model_version": "cs2-tiered-elo-v6", "observed_at_utc": "2026-10-13T22:29:07.911078+00:00", "probabilities": {"away": 0.51072, "home": 0.48928}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "908c3baddf4ba86217f65d4048d17d9e667ec4670b15f66a739c226d8f898288", "sport": "CS2"}</t>
+          <t>{"artifact_hash": "642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7", "away_team": "ex-RUSTEC", "event_id": "157864", "event_start_utc": "2026-10-14T17:00:00Z", "features": {"away_elo": 1787.204398, "away_history_count": 64, "home_elo": 1905.479513, "home_history_count": 64}, "historical_source_observation_times_verified": false, "home_team": "Black Phoenix", "inference_inputs": {"book_state": {"games_played": {"bo3:1:24857": 64, "bo3:1:24924": 64}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 40.0, "last_match_utc": {"bo3:1:24857": "2026-10-12T21:20:00Z", "bo3:1:24924": "2026-10-13T17:00:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.06821870672347567, "platt_slope": 0.8748911450799665, "ratings": {"bo3:1:24857": 1787.204398, "bo3:1:24924": 1905.479513}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "3abbfc5d7124cc94603dada2e4c996da231a679d437c5a066d994a2a7d428f61", "features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872"}, "reference_date": "2026-10-14T05:52:14.154858+00:00", "team_ids": ["bo3:1:24924", "bo3:1:24857"]}, "market_type": "moneyline", "model_version": "cs2-tiered-elo-v6", "observed_at_utc": "2026-10-14T05:52:14.154858+00:00", "probabilities": {"away": 0.361405, "home": 0.638595}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "898884aa76979a33708074a5c8f0cfc2fb21c63c7cc18dd52b74d46528e7650b", "sport": "CS2"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="36" customHeight="1">
+      <c r="A145" s="24" t="inlineStr">
+        <is>
+          <t>d51157ac9ae043a0</t>
+        </is>
+      </c>
+      <c r="B145" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-14T06:03:43.455911Z</t>
+        </is>
+      </c>
+      <c r="C145" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-14T19:00:00Z</t>
+        </is>
+      </c>
+      <c r="D145" s="24" t="inlineStr">
+        <is>
+          <t>157274</t>
+        </is>
+      </c>
+      <c r="E145" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F145" s="24" t="inlineStr">
+        <is>
+          <t>Alianza Lima Esports</t>
+        </is>
+      </c>
+      <c r="G145" s="24" t="inlineStr">
+        <is>
+          <t>Damajuana</t>
+        </is>
+      </c>
+      <c r="H145" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I145" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J145" s="25" t="n"/>
+      <c r="K145" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L145" s="26" t="n">
+        <v>108</v>
+      </c>
+      <c r="M145" s="27" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="N145" s="28" t="n">
+        <v>0.480769</v>
+      </c>
+      <c r="O145" s="28" t="n">
+        <v>0.618157</v>
+      </c>
+      <c r="P145" s="28" t="n"/>
+      <c r="Q145" s="28" t="n">
+        <v>0.137388</v>
+      </c>
+      <c r="R145" s="26" t="n">
+        <v>89</v>
+      </c>
+      <c r="S145" s="29" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="T145" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U145" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V145" s="24" t="n"/>
+      <c r="W145" s="26" t="n"/>
+      <c r="X145" s="26" t="n"/>
+      <c r="Y145" s="25" t="n"/>
+      <c r="Z145" s="26" t="n"/>
+      <c r="AA145" s="28" t="n"/>
+      <c r="AB145" s="28" t="n"/>
+      <c r="AC145" s="30" t="n"/>
+      <c r="AD145" s="24" t="n"/>
+      <c r="AE145" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.4800 (market_slug=aec-cs2-dam-ale-2026-10-14).</t>
+        </is>
+      </c>
+      <c r="AF145" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG145" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH145" s="24" t="n"/>
+      <c r="AI145" s="31" t="n"/>
+      <c r="AJ145" s="31" t="n"/>
+      <c r="AK145" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL145" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM145" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN145" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO145" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP145" s="24" t="inlineStr">
+        <is>
+          <t>Alianza Lima Esports</t>
+        </is>
+      </c>
+      <c r="AQ145" s="24" t="inlineStr">
+        <is>
+          <t>Alianza Lima Esports</t>
+        </is>
+      </c>
+      <c r="AR145" s="24" t="inlineStr">
+        <is>
+          <t>Alianza Lima Esports</t>
+        </is>
+      </c>
+      <c r="AS145" s="24" t="inlineStr">
+        <is>
+          <t>Damajuana</t>
+        </is>
+      </c>
+      <c r="AT145" s="24" t="inlineStr">
+        <is>
+          <t>Damajuana</t>
+        </is>
+      </c>
+      <c r="AU145" s="24" t="inlineStr">
+        <is>
+          <t>Damajuana</t>
+        </is>
+      </c>
+      <c r="AV145" s="24" t="n"/>
+      <c r="AW145" s="24" t="n"/>
+      <c r="AX145" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY145" s="24" t="n"/>
+      <c r="AZ145" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA145" s="24" t="inlineStr">
+        <is>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
+        </is>
+      </c>
+      <c r="BB145" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC145" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="BD145" s="24" t="inlineStr">
+        <is>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
+        </is>
+      </c>
+      <c r="BE145" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF145" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG145" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="BH145" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-14T06:02:19.213529Z</t>
+        </is>
+      </c>
+      <c r="BI145" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ145" s="25" t="n"/>
+      <c r="BK145" s="26" t="n">
+        <v>108</v>
+      </c>
+      <c r="BL145" s="27" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="BM145" s="28" t="n">
+        <v>0.480769</v>
+      </c>
+      <c r="BN145" s="28" t="n"/>
+      <c r="BO145" s="28" t="n"/>
+      <c r="BP145" s="25" t="n"/>
+      <c r="BQ145" s="27" t="n"/>
+      <c r="BR145" s="28" t="n"/>
+      <c r="BS145" s="28" t="n"/>
+      <c r="BT145" s="28" t="n"/>
+      <c r="BU145" s="25" t="n"/>
+      <c r="BV145" s="29" t="n"/>
+      <c r="BW145" s="24" t="n"/>
+      <c r="BX145" s="30" t="n"/>
+      <c r="BY145" s="27" t="n"/>
+      <c r="BZ145" s="24" t="n"/>
+      <c r="CA145" s="31" t="n"/>
+      <c r="CB145" s="24" t="n"/>
+      <c r="CC145" s="24" t="n"/>
+      <c r="CD145" s="24" t="n"/>
+      <c r="CE145" s="24" t="n"/>
+      <c r="CF145" s="24" t="n"/>
+      <c r="CG145" s="24" t="n"/>
+      <c r="CH145" s="24" t="n"/>
+      <c r="CI145" s="24" t="n"/>
+      <c r="CJ145" s="24" t="n"/>
+      <c r="CK145" s="24" t="n"/>
+      <c r="CL145" s="24" t="n"/>
+      <c r="CM145" s="24" t="n"/>
+      <c r="CN145" s="24" t="n"/>
+      <c r="CO145" s="24" t="n"/>
+      <c r="CP145" s="24" t="n"/>
+      <c r="CQ145" s="24" t="n"/>
+      <c r="CR145" s="24" t="n"/>
+      <c r="CS145" s="24" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CT145" s="24" t="n"/>
+      <c r="CU145" s="24" t="n"/>
+      <c r="CV145" s="24" t="n"/>
+      <c r="CW145" s="24" t="n"/>
+      <c r="CX145" s="24" t="n"/>
+      <c r="CY145" s="24" t="n"/>
+      <c r="CZ145" s="24" t="n"/>
+      <c r="DA145" s="24" t="n"/>
+      <c r="DB145" s="24" t="n"/>
+      <c r="DC145" s="24" t="n"/>
+      <c r="DD145" s="24" t="n"/>
+      <c r="DE145" s="24" t="n"/>
+      <c r="DF145" s="24" t="n"/>
+      <c r="DG145" s="24" t="n"/>
+      <c r="DH145" s="24" t="n"/>
+      <c r="DI145" s="24" t="n"/>
+      <c r="DJ145" s="24" t="n"/>
+      <c r="DK145" s="24" t="n"/>
+      <c r="DL145" s="24" t="n"/>
+      <c r="DM145" s="24" t="n"/>
+      <c r="DN145" s="24" t="n"/>
+      <c r="DO145" s="24" t="n"/>
+      <c r="DP145" s="24" t="n"/>
+      <c r="DQ145" s="24" t="inlineStr">
+        <is>
+          <t>{"artifact_hash": "642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7", "away_team": "Alianza Lima Esports", "event_id": "157274", "event_start_utc": "2026-10-14T19:00:00Z", "features": {"away_elo": 1385.592921, "away_history_count": 48, "home_elo": 1302.752503, "home_history_count": 17}, "historical_source_observation_times_verified": false, "home_team": "Damajuana", "inference_inputs": {"book_state": {"games_played": {"bo3:1:22881": 17, "bo3:1:4949": 48}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 40.0, "last_match_utc": {"bo3:1:22881": "2026-09-28T19:00:00Z", "bo3:1:4949": "2024-09-05T19:10:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.06821870672347567, "platt_slope": 0.8748911450799665, "ratings": {"bo3:1:22881": 1302.752503, "bo3:1:4949": 1385.592921}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "3abbfc5d7124cc94603dada2e4c996da231a679d437c5a066d994a2a7d428f61", "features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872"}, "reference_date": "2026-10-14T05:52:14.154858+00:00", "team_ids": ["bo3:1:22881", "bo3:1:4949"]}, "market_type": "moneyline", "model_version": "cs2-tiered-elo-v6", "observed_at_utc": "2026-10-14T05:52:14.154858+00:00", "probabilities": {"away": 0.618157, "home": 0.381843}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "4dca24d7f6c2e958d7a7b49840858bc1e09ea7201c50a4e847313fb02e9fa6c1", "sport": "CS2"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="36" customHeight="1">
+      <c r="A146" s="24" t="inlineStr">
+        <is>
+          <t>1f1bf9618b084c89</t>
+        </is>
+      </c>
+      <c r="B146" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-14T06:03:43.455911Z</t>
+        </is>
+      </c>
+      <c r="C146" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-14T19:00:00Z</t>
+        </is>
+      </c>
+      <c r="D146" s="24" t="inlineStr">
+        <is>
+          <t>157274</t>
+        </is>
+      </c>
+      <c r="E146" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F146" s="24" t="inlineStr">
+        <is>
+          <t>Alianza Lima Esports</t>
+        </is>
+      </c>
+      <c r="G146" s="24" t="inlineStr">
+        <is>
+          <t>Damajuana</t>
+        </is>
+      </c>
+      <c r="H146" s="24" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="I146" s="24" t="inlineStr">
+        <is>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="J146" s="25" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K146" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L146" s="26" t="n">
+        <v>-150</v>
+      </c>
+      <c r="M146" s="27" t="n">
+        <v>1.666667</v>
+      </c>
+      <c r="N146" s="28" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="O146" s="28" t="n">
+        <v>0.512621</v>
+      </c>
+      <c r="P146" s="28" t="n"/>
+      <c r="Q146" s="28" t="n">
+        <v>-0.087379</v>
+      </c>
+      <c r="R146" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="S146" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="T146" s="24" t="inlineStr">
+        <is>
+          <t>cs2-total-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U146" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V146" s="24" t="n"/>
+      <c r="W146" s="26" t="n"/>
+      <c r="X146" s="26" t="n"/>
+      <c r="Y146" s="25" t="n"/>
+      <c r="Z146" s="26" t="n"/>
+      <c r="AA146" s="28" t="n"/>
+      <c r="AB146" s="28" t="n"/>
+      <c r="AC146" s="30" t="n"/>
+      <c r="AD146" s="24" t="n"/>
+      <c r="AE146" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.6000 (market_slug=tsc-cs2-dam-ale-2026-10-14-tot-2pt5).</t>
+        </is>
+      </c>
+      <c r="AF146" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG146" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH146" s="24" t="n"/>
+      <c r="AI146" s="31" t="n"/>
+      <c r="AJ146" s="31" t="n"/>
+      <c r="AK146" s="24" t="inlineStr">
+        <is>
+          <t>paper_call</t>
+        </is>
+      </c>
+      <c r="AL146" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM146" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN146" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO146" s="24" t="inlineStr">
+        <is>
+          <t>PAPER_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP146" s="24" t="inlineStr">
+        <is>
+          <t>Alianza Lima Esports</t>
+        </is>
+      </c>
+      <c r="AQ146" s="24" t="inlineStr">
+        <is>
+          <t>Alianza Lima Esports</t>
+        </is>
+      </c>
+      <c r="AR146" s="24" t="inlineStr">
+        <is>
+          <t>Alianza Lima Esports</t>
+        </is>
+      </c>
+      <c r="AS146" s="24" t="inlineStr">
+        <is>
+          <t>Damajuana</t>
+        </is>
+      </c>
+      <c r="AT146" s="24" t="inlineStr">
+        <is>
+          <t>Damajuana</t>
+        </is>
+      </c>
+      <c r="AU146" s="24" t="inlineStr">
+        <is>
+          <t>Damajuana</t>
+        </is>
+      </c>
+      <c r="AV146" s="24" t="n"/>
+      <c r="AW146" s="24" t="n"/>
+      <c r="AX146" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY146" s="24" t="n"/>
+      <c r="AZ146" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA146" s="24" t="inlineStr">
+        <is>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
+        </is>
+      </c>
+      <c r="BB146" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC146" s="24" t="inlineStr">
+        <is>
+          <t>cs2-total-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="BD146" s="24" t="inlineStr">
+        <is>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
+        </is>
+      </c>
+      <c r="BE146" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF146" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG146" s="24" t="inlineStr">
+        <is>
+          <t>cs2-total-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="BH146" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-14T06:02:29.341277Z</t>
+        </is>
+      </c>
+      <c r="BI146" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ146" s="25" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="BK146" s="26" t="n">
+        <v>-150</v>
+      </c>
+      <c r="BL146" s="27" t="n">
+        <v>1.666667</v>
+      </c>
+      <c r="BM146" s="28" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="BN146" s="28" t="n"/>
+      <c r="BO146" s="28" t="n"/>
+      <c r="BP146" s="25" t="n"/>
+      <c r="BQ146" s="27" t="n"/>
+      <c r="BR146" s="28" t="n"/>
+      <c r="BS146" s="28" t="n"/>
+      <c r="BT146" s="28" t="n"/>
+      <c r="BU146" s="25" t="n"/>
+      <c r="BV146" s="29" t="n"/>
+      <c r="BW146" s="24" t="n"/>
+      <c r="BX146" s="30" t="n"/>
+      <c r="BY146" s="27" t="n"/>
+      <c r="BZ146" s="24" t="n"/>
+      <c r="CA146" s="31" t="n"/>
+      <c r="CB146" s="24" t="n"/>
+      <c r="CC146" s="24" t="n"/>
+      <c r="CD146" s="24" t="n"/>
+      <c r="CE146" s="24" t="n"/>
+      <c r="CF146" s="24" t="n"/>
+      <c r="CG146" s="24" t="n"/>
+      <c r="CH146" s="24" t="n"/>
+      <c r="CI146" s="24" t="n"/>
+      <c r="CJ146" s="24" t="n"/>
+      <c r="CK146" s="24" t="n"/>
+      <c r="CL146" s="24" t="n"/>
+      <c r="CM146" s="24" t="n"/>
+      <c r="CN146" s="24" t="n"/>
+      <c r="CO146" s="24" t="n"/>
+      <c r="CP146" s="24" t="n"/>
+      <c r="CQ146" s="24" t="n"/>
+      <c r="CR146" s="24" t="n"/>
+      <c r="CS146" s="24" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="CT146" s="24" t="n"/>
+      <c r="CU146" s="24" t="n"/>
+      <c r="CV146" s="24" t="n"/>
+      <c r="CW146" s="24" t="n"/>
+      <c r="CX146" s="24" t="n"/>
+      <c r="CY146" s="24" t="n"/>
+      <c r="CZ146" s="24" t="n"/>
+      <c r="DA146" s="24" t="n"/>
+      <c r="DB146" s="24" t="n"/>
+      <c r="DC146" s="24" t="n"/>
+      <c r="DD146" s="24" t="n"/>
+      <c r="DE146" s="24" t="n"/>
+      <c r="DF146" s="24" t="n"/>
+      <c r="DG146" s="24" t="n"/>
+      <c r="DH146" s="24" t="n"/>
+      <c r="DI146" s="24" t="n"/>
+      <c r="DJ146" s="24" t="n"/>
+      <c r="DK146" s="24" t="n"/>
+      <c r="DL146" s="24" t="n"/>
+      <c r="DM146" s="24" t="n"/>
+      <c r="DN146" s="24" t="n"/>
+      <c r="DO146" s="24" t="n"/>
+      <c r="DP146" s="24" t="n"/>
+      <c r="DQ146" s="24" t="n"/>
+    </row>
+    <row r="147" ht="36" customHeight="1">
+      <c r="A147" s="24" t="inlineStr">
+        <is>
+          <t>5fe62a57b5024cae</t>
+        </is>
+      </c>
+      <c r="B147" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-14T06:03:43.455911Z</t>
+        </is>
+      </c>
+      <c r="C147" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-14T21:00:00Z</t>
+        </is>
+      </c>
+      <c r="D147" s="24" t="inlineStr">
+        <is>
+          <t>159298</t>
+        </is>
+      </c>
+      <c r="E147" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F147" s="24" t="inlineStr">
+        <is>
+          <t>Galorys</t>
+        </is>
+      </c>
+      <c r="G147" s="24" t="inlineStr">
+        <is>
+          <t>largadosypelados</t>
+        </is>
+      </c>
+      <c r="H147" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I147" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J147" s="25" t="n"/>
+      <c r="K147" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L147" s="26" t="n">
+        <v>-122</v>
+      </c>
+      <c r="M147" s="27" t="n">
+        <v>1.819672</v>
+      </c>
+      <c r="N147" s="28" t="n">
+        <v>0.54955</v>
+      </c>
+      <c r="O147" s="28" t="n">
+        <v>0.636757</v>
+      </c>
+      <c r="P147" s="28" t="n"/>
+      <c r="Q147" s="28" t="n">
+        <v>0.08720700000000001</v>
+      </c>
+      <c r="R147" s="26" t="n">
+        <v>64</v>
+      </c>
+      <c r="S147" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T147" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U147" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V147" s="24" t="n"/>
+      <c r="W147" s="26" t="n"/>
+      <c r="X147" s="26" t="n"/>
+      <c r="Y147" s="25" t="n"/>
+      <c r="Z147" s="26" t="n"/>
+      <c r="AA147" s="28" t="n"/>
+      <c r="AB147" s="28" t="n"/>
+      <c r="AC147" s="30" t="n"/>
+      <c r="AD147" s="24" t="n"/>
+      <c r="AE147" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.5500 (market_slug=aec-cs2-ldp-gls-2026-10-14).</t>
+        </is>
+      </c>
+      <c r="AF147" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG147" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH147" s="24" t="n"/>
+      <c r="AI147" s="31" t="n"/>
+      <c r="AJ147" s="31" t="n"/>
+      <c r="AK147" s="24" t="inlineStr">
+        <is>
+          <t>paper_call</t>
+        </is>
+      </c>
+      <c r="AL147" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM147" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN147" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO147" s="24" t="inlineStr">
+        <is>
+          <t>PAPER_CALL_MODEL_UNVALIDATED</t>
+        </is>
+      </c>
+      <c r="AP147" s="24" t="inlineStr">
+        <is>
+          <t>Galorys</t>
+        </is>
+      </c>
+      <c r="AQ147" s="24" t="inlineStr">
+        <is>
+          <t>Galorys</t>
+        </is>
+      </c>
+      <c r="AR147" s="24" t="inlineStr">
+        <is>
+          <t>Galorys</t>
+        </is>
+      </c>
+      <c r="AS147" s="24" t="inlineStr">
+        <is>
+          <t>largadosypelados</t>
+        </is>
+      </c>
+      <c r="AT147" s="24" t="inlineStr">
+        <is>
+          <t>largadosypelados</t>
+        </is>
+      </c>
+      <c r="AU147" s="24" t="inlineStr">
+        <is>
+          <t>largadosypelados</t>
+        </is>
+      </c>
+      <c r="AV147" s="24" t="n"/>
+      <c r="AW147" s="24" t="n"/>
+      <c r="AX147" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY147" s="24" t="n"/>
+      <c r="AZ147" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA147" s="24" t="inlineStr">
+        <is>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
+        </is>
+      </c>
+      <c r="BB147" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC147" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="BD147" s="24" t="inlineStr">
+        <is>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
+        </is>
+      </c>
+      <c r="BE147" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF147" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG147" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="BH147" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-14T06:02:39.765904Z</t>
+        </is>
+      </c>
+      <c r="BI147" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ147" s="25" t="n"/>
+      <c r="BK147" s="26" t="n">
+        <v>-122</v>
+      </c>
+      <c r="BL147" s="27" t="n">
+        <v>1.819672</v>
+      </c>
+      <c r="BM147" s="28" t="n">
+        <v>0.54955</v>
+      </c>
+      <c r="BN147" s="28" t="n"/>
+      <c r="BO147" s="28" t="n"/>
+      <c r="BP147" s="25" t="n"/>
+      <c r="BQ147" s="27" t="n"/>
+      <c r="BR147" s="28" t="n"/>
+      <c r="BS147" s="28" t="n"/>
+      <c r="BT147" s="28" t="n"/>
+      <c r="BU147" s="25" t="n"/>
+      <c r="BV147" s="29" t="n"/>
+      <c r="BW147" s="24" t="n"/>
+      <c r="BX147" s="30" t="n"/>
+      <c r="BY147" s="27" t="n"/>
+      <c r="BZ147" s="24" t="n"/>
+      <c r="CA147" s="31" t="n"/>
+      <c r="CB147" s="24" t="n"/>
+      <c r="CC147" s="24" t="n"/>
+      <c r="CD147" s="24" t="n"/>
+      <c r="CE147" s="24" t="n"/>
+      <c r="CF147" s="24" t="n"/>
+      <c r="CG147" s="24" t="n"/>
+      <c r="CH147" s="24" t="n"/>
+      <c r="CI147" s="24" t="n"/>
+      <c r="CJ147" s="24" t="n"/>
+      <c r="CK147" s="24" t="n"/>
+      <c r="CL147" s="24" t="n"/>
+      <c r="CM147" s="24" t="n"/>
+      <c r="CN147" s="24" t="n"/>
+      <c r="CO147" s="24" t="n"/>
+      <c r="CP147" s="24" t="n"/>
+      <c r="CQ147" s="24" t="n"/>
+      <c r="CR147" s="24" t="n"/>
+      <c r="CS147" s="24" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CT147" s="24" t="n"/>
+      <c r="CU147" s="24" t="n"/>
+      <c r="CV147" s="24" t="n"/>
+      <c r="CW147" s="24" t="n"/>
+      <c r="CX147" s="24" t="n"/>
+      <c r="CY147" s="24" t="n"/>
+      <c r="CZ147" s="24" t="n"/>
+      <c r="DA147" s="24" t="n"/>
+      <c r="DB147" s="24" t="n"/>
+      <c r="DC147" s="24" t="n"/>
+      <c r="DD147" s="24" t="n"/>
+      <c r="DE147" s="24" t="n"/>
+      <c r="DF147" s="24" t="n"/>
+      <c r="DG147" s="24" t="n"/>
+      <c r="DH147" s="24" t="n"/>
+      <c r="DI147" s="24" t="n"/>
+      <c r="DJ147" s="24" t="n"/>
+      <c r="DK147" s="24" t="n"/>
+      <c r="DL147" s="24" t="n"/>
+      <c r="DM147" s="24" t="n"/>
+      <c r="DN147" s="24" t="n"/>
+      <c r="DO147" s="24" t="n"/>
+      <c r="DP147" s="24" t="n"/>
+      <c r="DQ147" s="24" t="inlineStr">
+        <is>
+          <t>{"artifact_hash": "642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7", "away_team": "Galorys", "event_id": "159298", "event_start_utc": "2026-10-14T21:00:00Z", "features": {"away_elo": 1802.356808, "away_history_count": 314, "home_elo": 1500.0, "home_history_count": 0}, "historical_source_observation_times_verified": false, "home_team": "largadosypelados", "inference_inputs": {"book_state": {"games_played": {"bo3:1:10049": 314}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 40.0, "last_match_utc": {"bo3:1:10049": "2026-10-13T21:00:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.06821870672347567, "platt_slope": 0.8748911450799665, "ratings": {"bo3:1:10049": 1802.356808}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "3abbfc5d7124cc94603dada2e4c996da231a679d437c5a066d994a2a7d428f61", "features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872"}, "reference_date": "2026-10-14T05:52:14.154858+00:00", "team_ids": ["unknown:largadosypelados", "bo3:1:10049"]}, "market_type": "moneyline", "model_version": "cs2-tiered-elo-v6", "observed_at_utc": "2026-10-14T05:52:14.154858+00:00", "probabilities": {"away": 0.636757, "home": 0.363243}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "14561daeca01b5ef0d5dc4bfbb5841bbd0dbe1d50f55a5fc10b81f8e4e5a4e47", "sport": "CS2"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="36" customHeight="1">
+      <c r="A148" s="24" t="inlineStr">
+        <is>
+          <t>7517e78dc2514a32</t>
+        </is>
+      </c>
+      <c r="B148" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-14T06:03:43.455911Z</t>
+        </is>
+      </c>
+      <c r="C148" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-15T10:00:00Z</t>
+        </is>
+      </c>
+      <c r="D148" s="24" t="inlineStr">
+        <is>
+          <t>156265</t>
+        </is>
+      </c>
+      <c r="E148" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F148" s="24" t="inlineStr">
+        <is>
+          <t>Envy</t>
+        </is>
+      </c>
+      <c r="G148" s="24" t="inlineStr">
+        <is>
+          <t>Heroic</t>
+        </is>
+      </c>
+      <c r="H148" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I148" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J148" s="25" t="n"/>
+      <c r="K148" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L148" s="26" t="n">
+        <v>-203</v>
+      </c>
+      <c r="M148" s="27" t="n">
+        <v>1.492611</v>
+      </c>
+      <c r="N148" s="28" t="n">
+        <v>0.669967</v>
+      </c>
+      <c r="O148" s="28" t="n">
+        <v>0.6878379999999999</v>
+      </c>
+      <c r="P148" s="28" t="n"/>
+      <c r="Q148" s="28" t="n">
+        <v>0.017871</v>
+      </c>
+      <c r="R148" s="26" t="n">
+        <v>29</v>
+      </c>
+      <c r="S148" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="T148" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U148" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V148" s="24" t="n"/>
+      <c r="W148" s="26" t="n"/>
+      <c r="X148" s="26" t="n"/>
+      <c r="Y148" s="25" t="n"/>
+      <c r="Z148" s="26" t="n"/>
+      <c r="AA148" s="28" t="n"/>
+      <c r="AB148" s="28" t="n"/>
+      <c r="AC148" s="30" t="n"/>
+      <c r="AD148" s="24" t="n"/>
+      <c r="AE148" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.6700 (market_slug=aec-cs2-hero-envy-2026-10-15).</t>
+        </is>
+      </c>
+      <c r="AF148" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG148" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH148" s="24" t="n"/>
+      <c r="AI148" s="31" t="n"/>
+      <c r="AJ148" s="31" t="n"/>
+      <c r="AK148" s="24" t="inlineStr">
+        <is>
+          <t>paper_call</t>
+        </is>
+      </c>
+      <c r="AL148" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM148" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN148" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO148" s="24" t="inlineStr">
+        <is>
+          <t>PAPER_CALL_MODEL_UNVALIDATED</t>
+        </is>
+      </c>
+      <c r="AP148" s="24" t="inlineStr">
+        <is>
+          <t>Envy</t>
+        </is>
+      </c>
+      <c r="AQ148" s="24" t="inlineStr">
+        <is>
+          <t>Envy</t>
+        </is>
+      </c>
+      <c r="AR148" s="24" t="inlineStr">
+        <is>
+          <t>Envy</t>
+        </is>
+      </c>
+      <c r="AS148" s="24" t="inlineStr">
+        <is>
+          <t>Heroic</t>
+        </is>
+      </c>
+      <c r="AT148" s="24" t="inlineStr">
+        <is>
+          <t>Heroic</t>
+        </is>
+      </c>
+      <c r="AU148" s="24" t="inlineStr">
+        <is>
+          <t>Heroic</t>
+        </is>
+      </c>
+      <c r="AV148" s="24" t="n"/>
+      <c r="AW148" s="24" t="n"/>
+      <c r="AX148" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY148" s="24" t="n"/>
+      <c r="AZ148" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA148" s="24" t="inlineStr">
+        <is>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
+        </is>
+      </c>
+      <c r="BB148" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC148" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="BD148" s="24" t="inlineStr">
+        <is>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
+        </is>
+      </c>
+      <c r="BE148" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF148" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG148" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="BH148" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-14T06:03:00.664293Z</t>
+        </is>
+      </c>
+      <c r="BI148" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ148" s="25" t="n"/>
+      <c r="BK148" s="26" t="n">
+        <v>-203</v>
+      </c>
+      <c r="BL148" s="27" t="n">
+        <v>1.492611</v>
+      </c>
+      <c r="BM148" s="28" t="n">
+        <v>0.669967</v>
+      </c>
+      <c r="BN148" s="28" t="n"/>
+      <c r="BO148" s="28" t="n"/>
+      <c r="BP148" s="25" t="n"/>
+      <c r="BQ148" s="27" t="n"/>
+      <c r="BR148" s="28" t="n"/>
+      <c r="BS148" s="28" t="n"/>
+      <c r="BT148" s="28" t="n"/>
+      <c r="BU148" s="25" t="n"/>
+      <c r="BV148" s="29" t="n"/>
+      <c r="BW148" s="24" t="n"/>
+      <c r="BX148" s="30" t="n"/>
+      <c r="BY148" s="27" t="n"/>
+      <c r="BZ148" s="24" t="n"/>
+      <c r="CA148" s="31" t="n"/>
+      <c r="CB148" s="24" t="n"/>
+      <c r="CC148" s="24" t="n"/>
+      <c r="CD148" s="24" t="n"/>
+      <c r="CE148" s="24" t="n"/>
+      <c r="CF148" s="24" t="n"/>
+      <c r="CG148" s="24" t="n"/>
+      <c r="CH148" s="24" t="n"/>
+      <c r="CI148" s="24" t="n"/>
+      <c r="CJ148" s="24" t="n"/>
+      <c r="CK148" s="24" t="n"/>
+      <c r="CL148" s="24" t="n"/>
+      <c r="CM148" s="24" t="n"/>
+      <c r="CN148" s="24" t="n"/>
+      <c r="CO148" s="24" t="n"/>
+      <c r="CP148" s="24" t="n"/>
+      <c r="CQ148" s="24" t="n"/>
+      <c r="CR148" s="24" t="n"/>
+      <c r="CS148" s="24" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CT148" s="24" t="n"/>
+      <c r="CU148" s="24" t="n"/>
+      <c r="CV148" s="24" t="n"/>
+      <c r="CW148" s="24" t="n"/>
+      <c r="CX148" s="24" t="n"/>
+      <c r="CY148" s="24" t="n"/>
+      <c r="CZ148" s="24" t="n"/>
+      <c r="DA148" s="24" t="n"/>
+      <c r="DB148" s="24" t="n"/>
+      <c r="DC148" s="24" t="n"/>
+      <c r="DD148" s="24" t="n"/>
+      <c r="DE148" s="24" t="n"/>
+      <c r="DF148" s="24" t="n"/>
+      <c r="DG148" s="24" t="n"/>
+      <c r="DH148" s="24" t="n"/>
+      <c r="DI148" s="24" t="n"/>
+      <c r="DJ148" s="24" t="n"/>
+      <c r="DK148" s="24" t="n"/>
+      <c r="DL148" s="24" t="n"/>
+      <c r="DM148" s="24" t="n"/>
+      <c r="DN148" s="24" t="n"/>
+      <c r="DO148" s="24" t="n"/>
+      <c r="DP148" s="24" t="n"/>
+      <c r="DQ148" s="24" t="inlineStr">
+        <is>
+          <t>{"artifact_hash": "642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7", "away_team": "Envy", "event_id": "156265", "event_start_utc": "2026-10-15T10:00:00Z", "features": {"away_elo": 1500.0, "away_history_count": 0, "home_elo": 2017.272002, "home_history_count": 259}, "historical_source_observation_times_verified": false, "home_team": "Heroic", "inference_inputs": {"book_state": {"games_played": {"bo3:1:759": 259}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 40.0, "last_match_utc": {"bo3:1:759": "2026-09-26T17:10:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.06821870672347567, "platt_slope": 0.8748911450799665, "ratings": {"bo3:1:759": 2017.272002}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "3abbfc5d7124cc94603dada2e4c996da231a679d437c5a066d994a2a7d428f61", "features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872"}, "reference_date": "2026-10-14T05:52:14.154858+00:00", "team_ids": ["bo3:1:759", "unknown:envy"]}, "market_type": "moneyline", "model_version": "cs2-tiered-elo-v6", "observed_at_utc": "2026-10-14T05:52:14.154858+00:00", "probabilities": {"away": 0.312162, "home": 0.687838}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "e78df2191356c9ef3a4a38bf26a1677355ec14a5e50754e8defd7764e64eb569", "sport": "CS2"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="36" customHeight="1">
+      <c r="A149" s="24" t="inlineStr">
+        <is>
+          <t>3e0a90fde5c3448a</t>
+        </is>
+      </c>
+      <c r="B149" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-14T06:03:43.455911Z</t>
+        </is>
+      </c>
+      <c r="C149" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-15T10:00:00Z</t>
+        </is>
+      </c>
+      <c r="D149" s="24" t="inlineStr">
+        <is>
+          <t>156266</t>
+        </is>
+      </c>
+      <c r="E149" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F149" s="24" t="inlineStr">
+        <is>
+          <t>BC.Game Esports</t>
+        </is>
+      </c>
+      <c r="G149" s="24" t="inlineStr">
+        <is>
+          <t>MIBR</t>
+        </is>
+      </c>
+      <c r="H149" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I149" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J149" s="25" t="n"/>
+      <c r="K149" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L149" s="26" t="n">
+        <v>-122</v>
+      </c>
+      <c r="M149" s="27" t="n">
+        <v>1.819672</v>
+      </c>
+      <c r="N149" s="28" t="n">
+        <v>0.54955</v>
+      </c>
+      <c r="O149" s="28" t="n">
+        <v>0.6712630000000001</v>
+      </c>
+      <c r="P149" s="28" t="n"/>
+      <c r="Q149" s="28" t="n">
+        <v>0.121713</v>
+      </c>
+      <c r="R149" s="26" t="n">
+        <v>81</v>
+      </c>
+      <c r="S149" s="29" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="T149" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U149" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V149" s="24" t="n"/>
+      <c r="W149" s="26" t="n"/>
+      <c r="X149" s="26" t="n"/>
+      <c r="Y149" s="25" t="n"/>
+      <c r="Z149" s="26" t="n"/>
+      <c r="AA149" s="28" t="n"/>
+      <c r="AB149" s="28" t="n"/>
+      <c r="AC149" s="30" t="n"/>
+      <c r="AD149" s="24" t="n"/>
+      <c r="AE149" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.5500 (market_slug=aec-cs2-mibr-bcg-2026-10-15).</t>
+        </is>
+      </c>
+      <c r="AF149" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG149" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH149" s="24" t="n"/>
+      <c r="AI149" s="31" t="n"/>
+      <c r="AJ149" s="31" t="n"/>
+      <c r="AK149" s="24" t="inlineStr">
+        <is>
+          <t>paper_call</t>
+        </is>
+      </c>
+      <c r="AL149" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM149" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN149" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO149" s="24" t="inlineStr">
+        <is>
+          <t>PAPER_CALL_MODEL_UNVALIDATED</t>
+        </is>
+      </c>
+      <c r="AP149" s="24" t="inlineStr">
+        <is>
+          <t>BC.Game Esports</t>
+        </is>
+      </c>
+      <c r="AQ149" s="24" t="inlineStr">
+        <is>
+          <t>BC.Game Esports</t>
+        </is>
+      </c>
+      <c r="AR149" s="24" t="inlineStr">
+        <is>
+          <t>BC.Game Esports</t>
+        </is>
+      </c>
+      <c r="AS149" s="24" t="inlineStr">
+        <is>
+          <t>MIBR</t>
+        </is>
+      </c>
+      <c r="AT149" s="24" t="inlineStr">
+        <is>
+          <t>MIBR</t>
+        </is>
+      </c>
+      <c r="AU149" s="24" t="inlineStr">
+        <is>
+          <t>MIBR</t>
+        </is>
+      </c>
+      <c r="AV149" s="24" t="n"/>
+      <c r="AW149" s="24" t="n"/>
+      <c r="AX149" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY149" s="24" t="n"/>
+      <c r="AZ149" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA149" s="24" t="inlineStr">
+        <is>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
+        </is>
+      </c>
+      <c r="BB149" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC149" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="BD149" s="24" t="inlineStr">
+        <is>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
+        </is>
+      </c>
+      <c r="BE149" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF149" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG149" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="BH149" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-14T06:03:00.774480Z</t>
+        </is>
+      </c>
+      <c r="BI149" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ149" s="25" t="n"/>
+      <c r="BK149" s="26" t="n">
+        <v>-122</v>
+      </c>
+      <c r="BL149" s="27" t="n">
+        <v>1.819672</v>
+      </c>
+      <c r="BM149" s="28" t="n">
+        <v>0.54955</v>
+      </c>
+      <c r="BN149" s="28" t="n"/>
+      <c r="BO149" s="28" t="n"/>
+      <c r="BP149" s="25" t="n"/>
+      <c r="BQ149" s="27" t="n"/>
+      <c r="BR149" s="28" t="n"/>
+      <c r="BS149" s="28" t="n"/>
+      <c r="BT149" s="28" t="n"/>
+      <c r="BU149" s="25" t="n"/>
+      <c r="BV149" s="29" t="n"/>
+      <c r="BW149" s="24" t="n"/>
+      <c r="BX149" s="30" t="n"/>
+      <c r="BY149" s="27" t="n"/>
+      <c r="BZ149" s="24" t="n"/>
+      <c r="CA149" s="31" t="n"/>
+      <c r="CB149" s="24" t="n"/>
+      <c r="CC149" s="24" t="n"/>
+      <c r="CD149" s="24" t="n"/>
+      <c r="CE149" s="24" t="n"/>
+      <c r="CF149" s="24" t="n"/>
+      <c r="CG149" s="24" t="n"/>
+      <c r="CH149" s="24" t="n"/>
+      <c r="CI149" s="24" t="n"/>
+      <c r="CJ149" s="24" t="n"/>
+      <c r="CK149" s="24" t="n"/>
+      <c r="CL149" s="24" t="n"/>
+      <c r="CM149" s="24" t="n"/>
+      <c r="CN149" s="24" t="n"/>
+      <c r="CO149" s="24" t="n"/>
+      <c r="CP149" s="24" t="n"/>
+      <c r="CQ149" s="24" t="n"/>
+      <c r="CR149" s="24" t="n"/>
+      <c r="CS149" s="24" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CT149" s="24" t="n"/>
+      <c r="CU149" s="24" t="n"/>
+      <c r="CV149" s="24" t="n"/>
+      <c r="CW149" s="24" t="n"/>
+      <c r="CX149" s="24" t="n"/>
+      <c r="CY149" s="24" t="n"/>
+      <c r="CZ149" s="24" t="n"/>
+      <c r="DA149" s="24" t="n"/>
+      <c r="DB149" s="24" t="n"/>
+      <c r="DC149" s="24" t="n"/>
+      <c r="DD149" s="24" t="n"/>
+      <c r="DE149" s="24" t="n"/>
+      <c r="DF149" s="24" t="n"/>
+      <c r="DG149" s="24" t="n"/>
+      <c r="DH149" s="24" t="n"/>
+      <c r="DI149" s="24" t="n"/>
+      <c r="DJ149" s="24" t="n"/>
+      <c r="DK149" s="24" t="n"/>
+      <c r="DL149" s="24" t="n"/>
+      <c r="DM149" s="24" t="n"/>
+      <c r="DN149" s="24" t="n"/>
+      <c r="DO149" s="24" t="n"/>
+      <c r="DP149" s="24" t="n"/>
+      <c r="DQ149" s="24" t="inlineStr">
+        <is>
+          <t>{"artifact_hash": "642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7", "away_team": "BC.Game Esports", "event_id": "156266", "event_start_utc": "2026-10-15T10:00:00Z", "features": {"away_elo": 1500.0, "away_history_count": 0, "home_elo": 1967.505379, "home_history_count": 279}, "historical_source_observation_times_verified": false, "home_team": "MIBR", "inference_inputs": {"book_state": {"games_played": {"bo3:1:755": 279}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 40.0, "last_match_utc": {"bo3:1:755": "2026-09-19T18:30:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.06821870672347567, "platt_slope": 0.8748911450799665, "ratings": {"bo3:1:755": 1967.505379}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "3abbfc5d7124cc94603dada2e4c996da231a679d437c5a066d994a2a7d428f61", "features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872"}, "reference_date": "2026-10-14T05:52:14.154858+00:00", "team_ids": ["bo3:1:755", "unknown:bcgameesports"]}, "market_type": "moneyline", "model_version": "cs2-tiered-elo-v6", "observed_at_utc": "2026-10-14T05:52:14.154858+00:00", "probabilities": {"away": 0.328737, "home": 0.671263}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "2ac5de770dcdb2bb79155f465f0136144b78276bad3aea5950fda45d528bc4f8", "sport": "CS2"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="36" customHeight="1">
+      <c r="A150" s="24" t="inlineStr">
+        <is>
+          <t>a31e55e0663c4650</t>
+        </is>
+      </c>
+      <c r="B150" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-14T06:03:43.455911Z</t>
+        </is>
+      </c>
+      <c r="C150" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-15T14:00:00Z</t>
+        </is>
+      </c>
+      <c r="D150" s="24" t="inlineStr">
+        <is>
+          <t>157867</t>
+        </is>
+      </c>
+      <c r="E150" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F150" s="24" t="inlineStr">
+        <is>
+          <t>Fire Flux Esports</t>
+        </is>
+      </c>
+      <c r="G150" s="24" t="inlineStr">
+        <is>
+          <t>Butterfly</t>
+        </is>
+      </c>
+      <c r="H150" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I150" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J150" s="25" t="n"/>
+      <c r="K150" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L150" s="26" t="n">
+        <v>163</v>
+      </c>
+      <c r="M150" s="27" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="N150" s="28" t="n">
+        <v>0.380228</v>
+      </c>
+      <c r="O150" s="28" t="n">
+        <v>0.543955</v>
+      </c>
+      <c r="P150" s="28" t="n"/>
+      <c r="Q150" s="28" t="n">
+        <v>0.163727</v>
+      </c>
+      <c r="R150" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="S150" s="29" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="T150" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U150" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V150" s="24" t="n"/>
+      <c r="W150" s="26" t="n"/>
+      <c r="X150" s="26" t="n"/>
+      <c r="Y150" s="25" t="n"/>
+      <c r="Z150" s="26" t="n"/>
+      <c r="AA150" s="28" t="n"/>
+      <c r="AB150" s="28" t="n"/>
+      <c r="AC150" s="30" t="n"/>
+      <c r="AD150" s="24" t="n"/>
+      <c r="AE150" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.3800 (market_slug=aec-cs2-btf-ff-2026-10-15).</t>
+        </is>
+      </c>
+      <c r="AF150" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG150" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH150" s="24" t="n"/>
+      <c r="AI150" s="31" t="n"/>
+      <c r="AJ150" s="31" t="n"/>
+      <c r="AK150" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL150" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM150" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN150" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO150" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP150" s="24" t="inlineStr">
+        <is>
+          <t>Fire Flux Esports</t>
+        </is>
+      </c>
+      <c r="AQ150" s="24" t="inlineStr">
+        <is>
+          <t>Fire Flux Esports</t>
+        </is>
+      </c>
+      <c r="AR150" s="24" t="inlineStr">
+        <is>
+          <t>Fire Flux Esports</t>
+        </is>
+      </c>
+      <c r="AS150" s="24" t="inlineStr">
+        <is>
+          <t>Butterfly</t>
+        </is>
+      </c>
+      <c r="AT150" s="24" t="inlineStr">
+        <is>
+          <t>Butterfly</t>
+        </is>
+      </c>
+      <c r="AU150" s="24" t="inlineStr">
+        <is>
+          <t>Butterfly</t>
+        </is>
+      </c>
+      <c r="AV150" s="24" t="n"/>
+      <c r="AW150" s="24" t="n"/>
+      <c r="AX150" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY150" s="24" t="n"/>
+      <c r="AZ150" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA150" s="24" t="inlineStr">
+        <is>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
+        </is>
+      </c>
+      <c r="BB150" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC150" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="BD150" s="24" t="inlineStr">
+        <is>
+          <t>642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7</t>
+        </is>
+      </c>
+      <c r="BE150" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF150" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG150" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="BH150" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-14T06:03:12.366588Z</t>
+        </is>
+      </c>
+      <c r="BI150" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ150" s="25" t="n"/>
+      <c r="BK150" s="26" t="n">
+        <v>163</v>
+      </c>
+      <c r="BL150" s="27" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="BM150" s="28" t="n">
+        <v>0.380228</v>
+      </c>
+      <c r="BN150" s="28" t="n"/>
+      <c r="BO150" s="28" t="n"/>
+      <c r="BP150" s="25" t="n"/>
+      <c r="BQ150" s="27" t="n"/>
+      <c r="BR150" s="28" t="n"/>
+      <c r="BS150" s="28" t="n"/>
+      <c r="BT150" s="28" t="n"/>
+      <c r="BU150" s="25" t="n"/>
+      <c r="BV150" s="29" t="n"/>
+      <c r="BW150" s="24" t="n"/>
+      <c r="BX150" s="30" t="n"/>
+      <c r="BY150" s="27" t="n"/>
+      <c r="BZ150" s="24" t="n"/>
+      <c r="CA150" s="31" t="n"/>
+      <c r="CB150" s="24" t="n"/>
+      <c r="CC150" s="24" t="n"/>
+      <c r="CD150" s="24" t="n"/>
+      <c r="CE150" s="24" t="n"/>
+      <c r="CF150" s="24" t="n"/>
+      <c r="CG150" s="24" t="n"/>
+      <c r="CH150" s="24" t="n"/>
+      <c r="CI150" s="24" t="n"/>
+      <c r="CJ150" s="24" t="n"/>
+      <c r="CK150" s="24" t="n"/>
+      <c r="CL150" s="24" t="n"/>
+      <c r="CM150" s="24" t="n"/>
+      <c r="CN150" s="24" t="n"/>
+      <c r="CO150" s="24" t="n"/>
+      <c r="CP150" s="24" t="n"/>
+      <c r="CQ150" s="24" t="n"/>
+      <c r="CR150" s="24" t="n"/>
+      <c r="CS150" s="24" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CT150" s="24" t="n"/>
+      <c r="CU150" s="24" t="n"/>
+      <c r="CV150" s="24" t="n"/>
+      <c r="CW150" s="24" t="n"/>
+      <c r="CX150" s="24" t="n"/>
+      <c r="CY150" s="24" t="n"/>
+      <c r="CZ150" s="24" t="n"/>
+      <c r="DA150" s="24" t="n"/>
+      <c r="DB150" s="24" t="n"/>
+      <c r="DC150" s="24" t="n"/>
+      <c r="DD150" s="24" t="n"/>
+      <c r="DE150" s="24" t="n"/>
+      <c r="DF150" s="24" t="n"/>
+      <c r="DG150" s="24" t="n"/>
+      <c r="DH150" s="24" t="n"/>
+      <c r="DI150" s="24" t="n"/>
+      <c r="DJ150" s="24" t="n"/>
+      <c r="DK150" s="24" t="n"/>
+      <c r="DL150" s="24" t="n"/>
+      <c r="DM150" s="24" t="n"/>
+      <c r="DN150" s="24" t="n"/>
+      <c r="DO150" s="24" t="n"/>
+      <c r="DP150" s="24" t="n"/>
+      <c r="DQ150" s="24" t="inlineStr">
+        <is>
+          <t>{"artifact_hash": "642b63c565f5bb5fd7361cee049bb5868e1ce2884480d212d2362f634573bdf7", "away_team": "Fire Flux Esports", "event_id": "157867", "event_start_utc": "2026-10-15T14:00:00Z", "features": {"away_elo": 1708.462113, "away_history_count": 323, "home_elo": 1660.985544, "home_history_count": 30}, "historical_source_observation_times_verified": false, "home_team": "Butterfly", "inference_inputs": {"book_state": {"games_played": {"bo3:1:16724": 323, "bo3:1:24855": 30}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 40.0, "last_match_utc": {"bo3:1:16724": "2026-10-12T11:10:00Z", "bo3:1:24855": "2026-10-06T14:00:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.06821870672347567, "platt_slope": 0.8748911450799665, "ratings": {"bo3:1:16724": 1708.462113, "bo3:1:24855": 1660.985544}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "3abbfc5d7124cc94603dada2e4c996da231a679d437c5a066d994a2a7d428f61", "features/elo_ratings.py": "d6513e79d65448c06cc0f9b9eed0eaa091567835128e1f6647a310da8d78a872"}, "reference_date": "2026-10-14T05:52:14.154858+00:00", "team_ids": ["bo3:1:24855", "bo3:1:16724"]}, "market_type": "moneyline", "model_version": "cs2-tiered-elo-v6", "observed_at_utc": "2026-10-14T05:52:14.154858+00:00", "probabilities": {"away": 0.543955, "home": 0.456045}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "11dffe620ef26ad97d25a99781761b196a191bc9b9630d4a6b138e754e810fac", "sport": "CS2"}</t>
         </is>
       </c>
     </row>

</xml_diff>